<commit_message>
Add Day 6 HDLBits reviews and FPGA dual-edge guide
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rb6ba222918824539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rf6abd2d8f2364f0f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -61,10 +61,10 @@
     <x:t xml:space="preserve">Day 5</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Pending</x:t>
+    <x:t xml:space="preserve">Day 6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Day 6</x:t>
+    <x:t xml:space="preserve">Pending</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Day 7</x:t>
@@ -136,7 +136,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -208,6 +208,16 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -247,7 +257,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -385,6 +395,30 @@
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -657,13 +691,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="1" t="n">
-        <x:v>85</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D3" s="1" t="n">
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
         <x:v>4</x:v>
@@ -1676,7 +1710,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E59" s="46" t="str">
-        <x:f>HYPERLINK("output/pdf/HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
+        <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
     </x:row>
@@ -2040,7 +2074,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E79" s="46" t="str">
-        <x:f>HYPERLINK("output/pdf/HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
+        <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
     </x:row>
@@ -2059,7 +2093,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E80" s="46" t="str">
-        <x:f>HYPERLINK("output/pdf/HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
+        <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
     </x:row>
@@ -2096,7 +2130,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E82" s="46" t="str">
-        <x:f>HYPERLINK("output/pdf/HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
+        <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
     </x:row>
@@ -2151,7 +2185,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E85" s="42" t="str">
-        <x:f>HYPERLINK("output/pdf/HDLBits_Entry80_Moore_Serial_Twos_Complement_Deep_Dive.pdf","Entry 80 Moore FSM PDF")</x:f>
+        <x:f>HYPERLINK("HDLBits_Entry80_Moore_Serial_Twos_Complement_Deep_Dive.pdf","Entry 80 Moore FSM PDF")</x:f>
         <x:v>Entry 80 Moore FSM PDF</x:v>
       </x:c>
     </x:row>
@@ -2261,10 +2295,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vectorr","Vector reversal 1")</x:f>
         <x:v>Vector reversal 1</x:v>
       </x:c>
-      <x:c r="D91" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E91" s="7"/>
+      <x:c r="D91" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E91" s="50" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="22.049999237060547" customHeight="1">
       <x:c r="A92" s="4">
@@ -2277,10 +2313,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dualedge","Dual-edge triggered flip-flop")</x:f>
         <x:v>Dual-edge triggered flip-flop</x:v>
       </x:c>
-      <x:c r="D92" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E92" s="7"/>
+      <x:c r="D92" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E92" s="54" t="str">
+        <x:f>HYPERLINK("HDLBits_Day6_Non_FSM_QA_Dualedge_and_Circuit5.pdf","Day 6 non-FSM Q&amp;A")</x:f>
+        <x:v>Day 6 non-FSM Q&amp;A</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="22.049999237060547" customHeight="1">
       <x:c r="A93" s="4">
@@ -2293,10 +2332,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/thermostat","Thermostat")</x:f>
         <x:v>Thermostat</x:v>
       </x:c>
-      <x:c r="D93" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E93" s="7"/>
+      <x:c r="D93" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E93" s="50" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="22.049999237060547" customHeight="1">
       <x:c r="A94" s="4">
@@ -2309,88 +2350,100 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit5","Combinational circuit 5")</x:f>
         <x:v>Combinational circuit 5</x:v>
       </x:c>
-      <x:c r="D94" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E94" s="7"/>
+      <x:c r="D94" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E94" s="54" t="str">
+        <x:f>HYPERLINK("HDLBits_Day6_Non_FSM_QA_Dualedge_and_Circuit5.pdf","Day 6 non-FSM Q&amp;A")</x:f>
+        <x:v>Day 6 non-FSM Q&amp;A</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="22.049999237060547" customHeight="1">
       <x:c r="A95" s="4">
         <x:v>90</x:v>
       </x:c>
       <x:c r="B95" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C95" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q3fsm","Q3a: FSM")</x:f>
         <x:v>Q3a: FSM</x:v>
       </x:c>
-      <x:c r="D95" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E95" s="7"/>
+      <x:c r="D95" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E95" s="54" t="str">
+        <x:f>HYPERLINK("HDLBits_Entry90_Exams_2014_Q3FSM_Three_Sample_Window_Deep_Dive.pdf","Q3FSM deep-dive PDF")</x:f>
+        <x:v>Q3FSM deep-dive PDF</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="22.049999237060547" customHeight="1">
       <x:c r="A96" s="4">
         <x:v>91</x:v>
       </x:c>
       <x:c r="B96" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C96" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector4","Replication operator")</x:f>
         <x:v>Replication operator</x:v>
       </x:c>
-      <x:c r="D96" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E96" s="7"/>
+      <x:c r="D96" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E96" s="50" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" ht="22.049999237060547" customHeight="1">
       <x:c r="A97" s="4">
         <x:v>92</x:v>
       </x:c>
       <x:c r="B97" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C97" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count15","Four-bit binary counter")</x:f>
         <x:v>Four-bit binary counter</x:v>
       </x:c>
-      <x:c r="D97" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E97" s="7"/>
+      <x:c r="D97" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E97" s="50" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="22.049999237060547" customHeight="1">
       <x:c r="A98" s="4">
         <x:v>93</x:v>
       </x:c>
       <x:c r="B98" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C98" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/popcount3","3-bit population count")</x:f>
         <x:v>3-bit population count</x:v>
       </x:c>
-      <x:c r="D98" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E98" s="7"/>
+      <x:c r="D98" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E98" s="50" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="22.049999237060547" customHeight="1">
       <x:c r="A99" s="4">
         <x:v>94</x:v>
       </x:c>
       <x:c r="B99" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C99" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gatesv","Gates and vectors")</x:f>
         <x:v>Gates and vectors</x:v>
       </x:c>
       <x:c r="D99" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E99" s="7"/>
     </x:row>
@@ -2399,14 +2452,14 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="B100" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C100" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count10","Decade counter")</x:f>
         <x:v>Decade counter</x:v>
       </x:c>
       <x:c r="D100" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E100" s="7"/>
     </x:row>
@@ -2415,14 +2468,14 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="B101" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C101" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector5","More replication")</x:f>
         <x:v>More replication</x:v>
       </x:c>
       <x:c r="D101" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E101" s="7"/>
     </x:row>
@@ -2431,14 +2484,14 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="B102" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C102" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q3bfsm","Q3b: FSM")</x:f>
         <x:v>Q3b: FSM</x:v>
       </x:c>
       <x:c r="D102" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E102" s="7"/>
     </x:row>
@@ -2447,14 +2500,14 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B103" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C103" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit6","Combinational circuit 6")</x:f>
         <x:v>Combinational circuit 6</x:v>
       </x:c>
       <x:c r="D103" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E103" s="7"/>
     </x:row>
@@ -2463,14 +2516,14 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="B104" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C104" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gatesv100","Even longer vectors")</x:f>
         <x:v>Even longer vectors</x:v>
       </x:c>
       <x:c r="D104" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E104" s="7"/>
     </x:row>
@@ -2479,14 +2532,14 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B105" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C105" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count1to10","Decade counter again")</x:f>
         <x:v>Decade counter again</x:v>
       </x:c>
       <x:c r="D105" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E105" s="7"/>
     </x:row>
@@ -2495,14 +2548,14 @@
         <x:v>101</x:v>
       </x:c>
       <x:c r="B106" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C106" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module","Modules")</x:f>
         <x:v>Modules</x:v>
       </x:c>
       <x:c r="D106" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E106" s="7"/>
     </x:row>
@@ -2511,14 +2564,14 @@
         <x:v>102</x:v>
       </x:c>
       <x:c r="B107" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C107" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q3c","Q3c: FSM logic")</x:f>
         <x:v>Q3c: FSM logic</x:v>
       </x:c>
       <x:c r="D107" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E107" s="7"/>
     </x:row>
@@ -2527,14 +2580,14 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="B108" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C108" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux2to1","2-to-1 multiplexer")</x:f>
         <x:v>2-to-1 multiplexer</x:v>
       </x:c>
       <x:c r="D108" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E108" s="7"/>
     </x:row>
@@ -2543,14 +2596,14 @@
         <x:v>104</x:v>
       </x:c>
       <x:c r="B109" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C109" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/countslow","Slow decade counter")</x:f>
         <x:v>Slow decade counter</x:v>
       </x:c>
       <x:c r="D109" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E109" s="7"/>
     </x:row>
@@ -2559,14 +2612,14 @@
         <x:v>105</x:v>
       </x:c>
       <x:c r="B110" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C110" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_pos","Connecting ports by position")</x:f>
         <x:v>Connecting ports by position</x:v>
       </x:c>
       <x:c r="D110" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E110" s="7"/>
     </x:row>
@@ -2575,14 +2628,14 @@
         <x:v>106</x:v>
       </x:c>
       <x:c r="B111" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C111" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit7","Sequential circuit 7")</x:f>
         <x:v>Sequential circuit 7</x:v>
       </x:c>
       <x:c r="D111" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E111" s="7"/>
     </x:row>
@@ -2591,14 +2644,14 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="B112" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C112" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q6b","Q6b: FSM next-state logic")</x:f>
         <x:v>Q6b: FSM next-state logic</x:v>
       </x:c>
       <x:c r="D112" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E112" s="7"/>
     </x:row>
@@ -2614,7 +2667,7 @@
         <x:v>2-to-1 bus multiplexer</x:v>
       </x:c>
       <x:c r="D113" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E113" s="7"/>
     </x:row>
@@ -2630,7 +2683,7 @@
         <x:v>Counter 1-12</x:v>
       </x:c>
       <x:c r="D114" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E114" s="7"/>
     </x:row>
@@ -2646,7 +2699,7 @@
         <x:v>Connecting ports by name</x:v>
       </x:c>
       <x:c r="D115" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E115" s="7"/>
     </x:row>
@@ -2662,7 +2715,7 @@
         <x:v>9-to-1 multiplexer</x:v>
       </x:c>
       <x:c r="D116" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E116" s="7"/>
     </x:row>
@@ -2678,7 +2731,7 @@
         <x:v>Q6c: FSM one-hot next-state logic</x:v>
       </x:c>
       <x:c r="D117" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E117" s="7"/>
     </x:row>
@@ -2694,7 +2747,7 @@
         <x:v>Counter 1000</x:v>
       </x:c>
       <x:c r="D118" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E118" s="7"/>
     </x:row>
@@ -2710,7 +2763,7 @@
         <x:v>Sequential circuit 8</x:v>
       </x:c>
       <x:c r="D119" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E119" s="7"/>
     </x:row>
@@ -2726,7 +2779,7 @@
         <x:v>256-to-1 multiplexer</x:v>
       </x:c>
       <x:c r="D120" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E120" s="7"/>
     </x:row>
@@ -2742,7 +2795,7 @@
         <x:v>Three modules</x:v>
       </x:c>
       <x:c r="D121" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E121" s="7"/>
     </x:row>
@@ -2758,7 +2811,7 @@
         <x:v>Q6: FSM</x:v>
       </x:c>
       <x:c r="D122" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E122" s="7"/>
     </x:row>
@@ -2774,7 +2827,7 @@
         <x:v>4-digit decimal counter</x:v>
       </x:c>
       <x:c r="D123" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E123" s="7"/>
     </x:row>
@@ -2790,7 +2843,7 @@
         <x:v>256-to-1 4-bit multiplexer</x:v>
       </x:c>
       <x:c r="D124" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E124" s="7"/>
     </x:row>
@@ -2806,7 +2859,7 @@
         <x:v>Modules and vectors</x:v>
       </x:c>
       <x:c r="D125" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E125" s="7"/>
     </x:row>
@@ -2822,7 +2875,7 @@
         <x:v>Sequential circuit 9</x:v>
       </x:c>
       <x:c r="D126" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E126" s="7"/>
     </x:row>
@@ -2838,7 +2891,7 @@
         <x:v>Half adder</x:v>
       </x:c>
       <x:c r="D127" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E127" s="7"/>
     </x:row>
@@ -2854,7 +2907,7 @@
         <x:v>12-hour clock</x:v>
       </x:c>
       <x:c r="D128" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E128" s="7"/>
     </x:row>
@@ -2870,7 +2923,7 @@
         <x:v>Q2a: FSM</x:v>
       </x:c>
       <x:c r="D129" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E129" s="7"/>
     </x:row>
@@ -2886,7 +2939,7 @@
         <x:v>Adder 1</x:v>
       </x:c>
       <x:c r="D130" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E130" s="7"/>
     </x:row>
@@ -2902,7 +2955,7 @@
         <x:v>Full adder</x:v>
       </x:c>
       <x:c r="D131" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E131" s="7"/>
     </x:row>
@@ -2918,7 +2971,7 @@
         <x:v>4-bit shift register</x:v>
       </x:c>
       <x:c r="D132" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E132" s="7"/>
     </x:row>
@@ -2934,7 +2987,7 @@
         <x:v>Q2b: One-hot FSM equations</x:v>
       </x:c>
       <x:c r="D133" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E133" s="7"/>
     </x:row>
@@ -2950,7 +3003,7 @@
         <x:v>Adder 2</x:v>
       </x:c>
       <x:c r="D134" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E134" s="7"/>
     </x:row>
@@ -2966,7 +3019,7 @@
         <x:v>3-bit binary adder</x:v>
       </x:c>
       <x:c r="D135" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E135" s="7"/>
     </x:row>
@@ -2982,7 +3035,7 @@
         <x:v>Left/right rotator</x:v>
       </x:c>
       <x:c r="D136" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E136" s="7"/>
     </x:row>
@@ -2998,7 +3051,7 @@
         <x:v>Sequential circuit 10</x:v>
       </x:c>
       <x:c r="D137" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E137" s="7"/>
     </x:row>
@@ -3014,7 +3067,7 @@
         <x:v>Q2a: FSM</x:v>
       </x:c>
       <x:c r="D138" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E138" s="7"/>
     </x:row>
@@ -3030,7 +3083,7 @@
         <x:v>Carry-select adder</x:v>
       </x:c>
       <x:c r="D139" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E139" s="7"/>
     </x:row>
@@ -3046,7 +3099,7 @@
         <x:v>Adder</x:v>
       </x:c>
       <x:c r="D140" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E140" s="7"/>
     </x:row>
@@ -3062,7 +3115,7 @@
         <x:v>Left/right arithmetic shift by 1 or 8</x:v>
       </x:c>
       <x:c r="D141" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E141" s="7"/>
     </x:row>
@@ -3078,7 +3131,7 @@
         <x:v>Signed addition overflow</x:v>
       </x:c>
       <x:c r="D142" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E142" s="7"/>
     </x:row>
@@ -3094,7 +3147,7 @@
         <x:v>Adder-subtractor</x:v>
       </x:c>
       <x:c r="D143" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E143" s="7"/>
     </x:row>
@@ -3110,7 +3163,7 @@
         <x:v>Q2b: Another FSM</x:v>
       </x:c>
       <x:c r="D144" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E144" s="7"/>
     </x:row>
@@ -3126,7 +3179,7 @@
         <x:v>Clock</x:v>
       </x:c>
       <x:c r="D145" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E145" s="7"/>
     </x:row>
@@ -3142,7 +3195,7 @@
         <x:v>5-bit LFSR</x:v>
       </x:c>
       <x:c r="D146" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E146" s="7"/>
     </x:row>
@@ -3158,7 +3211,7 @@
         <x:v>100-bit binary adder</x:v>
       </x:c>
       <x:c r="D147" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E147" s="7"/>
     </x:row>
@@ -3174,7 +3227,7 @@
         <x:v>Always blocks (combinational)</x:v>
       </x:c>
       <x:c r="D148" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E148" s="7"/>
     </x:row>
@@ -3190,7 +3243,7 @@
         <x:v>Counter with period 1000</x:v>
       </x:c>
       <x:c r="D149" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E149" s="7"/>
     </x:row>
@@ -3206,7 +3259,7 @@
         <x:v>3-bit LFSR</x:v>
       </x:c>
       <x:c r="D150" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E150" s="7"/>
     </x:row>
@@ -3222,7 +3275,7 @@
         <x:v>4-digit BCD adder</x:v>
       </x:c>
       <x:c r="D151" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E151" s="7"/>
     </x:row>
@@ -3238,7 +3291,7 @@
         <x:v>Always blocks (clocked)</x:v>
       </x:c>
       <x:c r="D152" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E152" s="7"/>
     </x:row>
@@ -3254,7 +3307,7 @@
         <x:v>Testbench1</x:v>
       </x:c>
       <x:c r="D153" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E153" s="7"/>
     </x:row>
@@ -3270,7 +3323,7 @@
         <x:v>4-bit shift register and down counter</x:v>
       </x:c>
       <x:c r="D154" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E154" s="7"/>
     </x:row>
@@ -3286,7 +3339,7 @@
         <x:v>3-variable</x:v>
       </x:c>
       <x:c r="D155" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E155" s="7"/>
     </x:row>
@@ -3302,7 +3355,7 @@
         <x:v>32-bit LFSR</x:v>
       </x:c>
       <x:c r="D156" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E156" s="7"/>
     </x:row>
@@ -3318,7 +3371,7 @@
         <x:v>If statement</x:v>
       </x:c>
       <x:c r="D157" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E157" s="7"/>
     </x:row>
@@ -3334,7 +3387,7 @@
         <x:v>4-variable</x:v>
       </x:c>
       <x:c r="D158" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E158" s="7"/>
     </x:row>
@@ -3350,7 +3403,7 @@
         <x:v>Shift register</x:v>
       </x:c>
       <x:c r="D159" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E159" s="7"/>
     </x:row>
@@ -3366,7 +3419,7 @@
         <x:v>FSM: Sequence 1101 recognizer</x:v>
       </x:c>
       <x:c r="D160" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E160" s="7"/>
     </x:row>
@@ -3382,7 +3435,7 @@
         <x:v>AND gate</x:v>
       </x:c>
       <x:c r="D161" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E161" s="7"/>
     </x:row>
@@ -3398,7 +3451,7 @@
         <x:v>4-variable</x:v>
       </x:c>
       <x:c r="D162" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E162" s="7"/>
     </x:row>
@@ -3414,7 +3467,7 @@
         <x:v>If statement latches</x:v>
       </x:c>
       <x:c r="D163" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E163" s="7"/>
     </x:row>
@@ -3430,7 +3483,7 @@
         <x:v>Shift register</x:v>
       </x:c>
       <x:c r="D164" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E164" s="7"/>
     </x:row>
@@ -3446,7 +3499,7 @@
         <x:v>FSM: Enable shift register</x:v>
       </x:c>
       <x:c r="D165" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E165" s="7"/>
     </x:row>
@@ -3462,7 +3515,7 @@
         <x:v>4-variable</x:v>
       </x:c>
       <x:c r="D166" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E166" s="7"/>
     </x:row>
@@ -3478,7 +3531,7 @@
         <x:v>Case statement</x:v>
       </x:c>
       <x:c r="D167" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E167" s="7"/>
     </x:row>
@@ -3494,7 +3547,7 @@
         <x:v>3-input LUT</x:v>
       </x:c>
       <x:c r="D168" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E168" s="7"/>
     </x:row>
@@ -3510,7 +3563,7 @@
         <x:v>Minimum SOP and POS</x:v>
       </x:c>
       <x:c r="D169" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E169" s="7"/>
     </x:row>
@@ -3526,7 +3579,7 @@
         <x:v>FSM: The complete FSM</x:v>
       </x:c>
       <x:c r="D170" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E170" s="7"/>
     </x:row>
@@ -3542,7 +3595,7 @@
         <x:v>Testbench2</x:v>
       </x:c>
       <x:c r="D171" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E171" s="7"/>
     </x:row>
@@ -3558,7 +3611,7 @@
         <x:v>Priority encoder</x:v>
       </x:c>
       <x:c r="D172" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E172" s="7"/>
     </x:row>
@@ -3574,7 +3627,7 @@
         <x:v>Rule 90</x:v>
       </x:c>
       <x:c r="D173" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E173" s="7"/>
     </x:row>
@@ -3590,7 +3643,7 @@
         <x:v>Karnaugh map</x:v>
       </x:c>
       <x:c r="D174" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E174" s="7"/>
     </x:row>
@@ -3606,7 +3659,7 @@
         <x:v>The complete timer</x:v>
       </x:c>
       <x:c r="D175" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E175" s="7"/>
     </x:row>
@@ -3622,7 +3675,7 @@
         <x:v>Priority encoder with casez</x:v>
       </x:c>
       <x:c r="D176" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E176" s="7"/>
     </x:row>
@@ -3638,7 +3691,7 @@
         <x:v>Rule 110</x:v>
       </x:c>
       <x:c r="D177" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E177" s="7"/>
     </x:row>
@@ -3654,7 +3707,7 @@
         <x:v>Karnaugh map</x:v>
       </x:c>
       <x:c r="D178" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E178" s="7"/>
     </x:row>
@@ -3670,7 +3723,7 @@
         <x:v>T flip-flop</x:v>
       </x:c>
       <x:c r="D179" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E179" s="7"/>
     </x:row>
@@ -3686,7 +3739,7 @@
         <x:v>FSM: One-hot logic equations</x:v>
       </x:c>
       <x:c r="D180" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E180" s="7"/>
     </x:row>
@@ -3702,7 +3755,7 @@
         <x:v>Avoiding latches</x:v>
       </x:c>
       <x:c r="D181" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E181" s="7"/>
     </x:row>
@@ -3718,7 +3771,7 @@
         <x:v>Conway's Game of Life 16x16</x:v>
       </x:c>
       <x:c r="D182" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E182" s="7"/>
     </x:row>
@@ -3734,7 +3787,7 @@
         <x:v>K-map implemented with a multiplexer</x:v>
       </x:c>
       <x:c r="D183" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E183" s="8"/>
     </x:row>
@@ -3758,7 +3811,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76c37173e21f49ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f73f4956c7e4a50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update Attempt 2 tracker through grouped Day 7 problems
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rf6abd2d8f2364f0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R8847ae000aab4e4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -64,10 +64,10 @@
     <x:t xml:space="preserve">Day 6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Pending</x:t>
+    <x:t xml:space="preserve">Day 7</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Day 7</x:t>
+    <x:t xml:space="preserve">Pending</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Day 8</x:t>
@@ -83,7 +83,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="10">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -122,21 +122,11 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF5B2C83"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
       <x:color rgb="FF0563C1"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF9E480E"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -218,6 +208,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -257,7 +252,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -289,137 +284,59 @@
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -669,35 +586,35 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28.950000762939453" customHeight="1">
-      <x:c r="A1" s="18" t="s">
+      <x:c r="A1" s="27" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="18"/>
-      <x:c r="C1" s="18"/>
-      <x:c r="D1" s="18"/>
-      <x:c r="E1" s="18"/>
+      <x:c r="B1" s="27"/>
+      <x:c r="C1" s="27"/>
+      <x:c r="D1" s="27"/>
+      <x:c r="E1" s="27"/>
     </x:row>
     <x:row r="2" ht="22.950000762939453" customHeight="1">
-      <x:c r="A2" s="19" t="s">
+      <x:c r="A2" s="28" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="19"/>
-      <x:c r="C2" s="19"/>
-      <x:c r="D2" s="19"/>
-      <x:c r="E2" s="19"/>
+      <x:c r="B2" s="28"/>
+      <x:c r="C2" s="28"/>
+      <x:c r="D2" s="28"/>
+      <x:c r="E2" s="28"/>
     </x:row>
     <x:row r="3" ht="25.049999237060547" customHeight="1">
       <x:c r="A3" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="1" t="n">
-        <x:v>93</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D3" s="1" t="n">
-        <x:v>85</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
         <x:v>4</x:v>
@@ -727,7 +644,7 @@
       <x:c r="B6" s="3" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lemmings1","Lemmings 1")</x:f>
         <x:v>Lemmings 1</x:v>
       </x:c>
@@ -745,14 +662,14 @@
       <x:c r="B7" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C7" s="13" t="str">
+      <x:c r="C7" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_serial","Serial receiver")</x:f>
         <x:v>Serial receiver</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E7" s="36" t="str">
+      <x:c r="E7" s="14" t="str">
         <x:f>HYPERLINK("HDLBits_Fsm_serialdata_For_Loops_vs_Clock_Cycles.pdf","Serial discussion PDF")</x:f>
         <x:v>Serial discussion PDF</x:v>
       </x:c>
@@ -764,7 +681,7 @@
       <x:c r="B8" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C8" s="13" t="str">
+      <x:c r="C8" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lemmings2","Lemmings 2")</x:f>
         <x:v>Lemmings 2</x:v>
       </x:c>
@@ -782,14 +699,14 @@
       <x:c r="B9" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C9" s="13" t="str">
+      <x:c r="C9" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_serialdata","Serial receiver and datapath")</x:f>
         <x:v>Serial receiver and datapath</x:v>
       </x:c>
       <x:c r="D9" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E9" s="36" t="str">
+      <x:c r="E9" s="14" t="str">
         <x:f>HYPERLINK("HDLBits_Fsm_serialdata_For_Loops_vs_Clock_Cycles.pdf","Serial discussion PDF")</x:f>
         <x:v>Serial discussion PDF</x:v>
       </x:c>
@@ -801,7 +718,7 @@
       <x:c r="B10" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C10" s="13" t="str">
+      <x:c r="C10" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lemmings3","Lemmings 3")</x:f>
         <x:v>Lemmings 3</x:v>
       </x:c>
@@ -819,14 +736,14 @@
       <x:c r="B11" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C11" s="13" t="str">
+      <x:c r="C11" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_serialdp","Serial receiver with parity checking")</x:f>
         <x:v>Serial receiver with parity checking</x:v>
       </x:c>
       <x:c r="D11" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E11" s="36" t="str">
+      <x:c r="E11" s="14" t="str">
         <x:f>HYPERLINK("HDLBits_Fsm_serialdata_For_Loops_vs_Clock_Cycles.pdf","Serial discussion PDF")</x:f>
         <x:v>Serial discussion PDF</x:v>
       </x:c>
@@ -838,14 +755,14 @@
       <x:c r="B12" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C12" s="13" t="str">
+      <x:c r="C12" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lemmings4","Lemmings 4")</x:f>
         <x:v>Lemmings 4</x:v>
       </x:c>
       <x:c r="D12" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E12" s="37" t="str">
+      <x:c r="E12" s="19" t="str">
         <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
         <x:v>Combined questions PDF</x:v>
       </x:c>
@@ -857,14 +774,14 @@
       <x:c r="B13" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C13" s="13" t="str">
+      <x:c r="C13" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_hdlc","Sequence recognition")</x:f>
         <x:v>Sequence recognition</x:v>
       </x:c>
       <x:c r="D13" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E13" s="38" t="str">
+      <x:c r="E13" s="20" t="str">
         <x:f>HYPERLINK("HDLBits_Fsm_hdlc_Mealy_to_Moore_Deep_Dive.pdf","HDLC discussion PDF")</x:f>
         <x:v>HDLC discussion PDF</x:v>
       </x:c>
@@ -876,7 +793,7 @@
       <x:c r="B14" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C14" s="13" t="str">
+      <x:c r="C14" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/conditional","Conditional ternary operator")</x:f>
         <x:v>Conditional ternary operator</x:v>
       </x:c>
@@ -894,7 +811,7 @@
       <x:c r="B15" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C15" s="13" t="str">
+      <x:c r="C15" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dff","D flip-flop")</x:f>
         <x:v>D flip-flop</x:v>
       </x:c>
@@ -912,7 +829,7 @@
       <x:c r="B16" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="13" t="str">
+      <x:c r="C16" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/step_one","Getting Started")</x:f>
         <x:v>Getting Started</x:v>
       </x:c>
@@ -930,7 +847,7 @@
       <x:c r="B17" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C17" s="13" t="str">
+      <x:c r="C17" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm1","Simple FSM 1 (asynchronous reset)")</x:f>
         <x:v>Simple FSM 1 (asynchronous reset)</x:v>
       </x:c>
@@ -948,14 +865,14 @@
       <x:c r="B18" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C18" s="13" t="str">
+      <x:c r="C18" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bugs_mux2","Mux")</x:f>
         <x:v>Mux</x:v>
       </x:c>
       <x:c r="D18" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E18" s="37" t="str">
+      <x:c r="E18" s="19" t="str">
         <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
         <x:v>Combined questions PDF</x:v>
       </x:c>
@@ -967,7 +884,7 @@
       <x:c r="B19" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C19" s="13" t="str">
+      <x:c r="C19" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/reduction","Reduction operators")</x:f>
         <x:v>Reduction operators</x:v>
       </x:c>
@@ -985,7 +902,7 @@
       <x:c r="B20" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C20" s="13" t="str">
+      <x:c r="C20" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dff8","D flip-flops")</x:f>
         <x:v>D flip-flops</x:v>
       </x:c>
@@ -1003,7 +920,7 @@
       <x:c r="B21" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="str">
+      <x:c r="C21" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/zero","Output Zero")</x:f>
         <x:v>Output Zero</x:v>
       </x:c>
@@ -1021,7 +938,7 @@
       <x:c r="B22" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C22" s="13" t="str">
+      <x:c r="C22" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm1s","Simple FSM 1 (synchronous reset)")</x:f>
         <x:v>Simple FSM 1 (synchronous reset)</x:v>
       </x:c>
@@ -1039,7 +956,7 @@
       <x:c r="B23" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C23" s="13" t="str">
+      <x:c r="C23" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gates100","Reduction: Even wider gates")</x:f>
         <x:v>Reduction: Even wider gates</x:v>
       </x:c>
@@ -1057,16 +974,16 @@
       <x:c r="B24" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C24" s="13" t="str">
+      <x:c r="C24" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dff8r","DFF with reset")</x:f>
         <x:v>DFF with reset</x:v>
       </x:c>
       <x:c r="D24" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E24" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
-        <x:v>Combined questions PDF</x:v>
+      <x:c r="E24" s="21" t="e">
+        <x:f t="shared" ref="E24:E36" si="0">HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=HDLBits_Combined_Questions_and_Day2_Review.pdf, friendlyName=Combined questions PDF</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="22.049999237060547" customHeight="1">
@@ -1076,15 +993,15 @@
       <x:c r="B25" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C25" s="13" t="str">
+      <x:c r="C25" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/wire","Simple wire")</x:f>
         <x:v>Simple wire</x:v>
       </x:c>
       <x:c r="D25" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E25" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E25" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1095,15 +1012,15 @@
       <x:c r="B26" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C26" s="13" t="str">
+      <x:c r="C26" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bugs_nand3","NAND")</x:f>
         <x:v>NAND</x:v>
       </x:c>
       <x:c r="D26" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E26" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E26" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1114,15 +1031,15 @@
       <x:c r="B27" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C27" s="13" t="str">
+      <x:c r="C27" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm2","Simple FSM 2 (asynchronous reset)")</x:f>
         <x:v>Simple FSM 2 (asynchronous reset)</x:v>
       </x:c>
       <x:c r="D27" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E27" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E27" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1133,15 +1050,15 @@
       <x:c r="B28" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C28" s="13" t="str">
+      <x:c r="C28" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector100r","Combinational for-loop: Vector reversal 2")</x:f>
         <x:v>Combinational for-loop: Vector reversal 2</x:v>
       </x:c>
       <x:c r="D28" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E28" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E28" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1152,15 +1069,15 @@
       <x:c r="B29" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C29" s="13" t="str">
+      <x:c r="C29" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dff8p","DFF with reset value")</x:f>
         <x:v>DFF with reset value</x:v>
       </x:c>
       <x:c r="D29" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E29" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E29" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1171,15 +1088,15 @@
       <x:c r="B30" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C30" s="13" t="str">
+      <x:c r="C30" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/wire4","Four wires")</x:f>
         <x:v>Four wires</x:v>
       </x:c>
       <x:c r="D30" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E30" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E30" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1190,15 +1107,15 @@
       <x:c r="B31" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C31" s="13" t="str">
+      <x:c r="C31" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/popcount255","Combinational for-loop: 255-bit population count")</x:f>
         <x:v>Combinational for-loop: 255-bit population count</x:v>
       </x:c>
       <x:c r="D31" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E31" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E31" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1209,15 +1126,15 @@
       <x:c r="B32" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C32" s="13" t="str">
+      <x:c r="C32" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm2s","Simple FSM 2 (synchronous reset)")</x:f>
         <x:v>Simple FSM 2 (synchronous reset)</x:v>
       </x:c>
       <x:c r="D32" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E32" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E32" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1228,15 +1145,15 @@
       <x:c r="B33" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C33" s="13" t="str">
+      <x:c r="C33" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dff8ar","DFF with asynchronous reset")</x:f>
         <x:v>DFF with asynchronous reset</x:v>
       </x:c>
       <x:c r="D33" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E33" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E33" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1247,15 +1164,15 @@
       <x:c r="B34" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C34" s="13" t="str">
+      <x:c r="C34" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bugs_mux4","Mux")</x:f>
         <x:v>Mux</x:v>
       </x:c>
       <x:c r="D34" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E34" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E34" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1266,15 +1183,15 @@
       <x:c r="B35" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C35" s="13" t="str">
+      <x:c r="C35" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/adder100i","Generate for-loop: 100-bit binary adder 2")</x:f>
         <x:v>Generate for-loop: 100-bit binary adder 2</x:v>
       </x:c>
       <x:c r="D35" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E35" s="39" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E35" s="21" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1292,8 +1209,8 @@
       <x:c r="D36" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E36" s="40" t="str">
-        <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
+      <x:c r="E36" s="6" t="str">
+        <x:f t="shared" si="0"/>
         <x:v>Combined questions PDF</x:v>
       </x:c>
     </x:row>
@@ -1322,7 +1239,7 @@
       <x:c r="B38" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C38" s="13" t="str">
+      <x:c r="C38" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dff16e","DFF with byte enable")</x:f>
         <x:v>DFF with byte enable</x:v>
       </x:c>
@@ -1340,7 +1257,7 @@
       <x:c r="B39" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C39" s="13" t="str">
+      <x:c r="C39" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bcdadd100","Generate for-loop: 100-digit BCD adder")</x:f>
         <x:v>Generate for-loop: 100-digit BCD adder</x:v>
       </x:c>
@@ -1358,7 +1275,7 @@
       <x:c r="B40" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C40" s="13" t="str">
+      <x:c r="C40" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/andgate","AND gate")</x:f>
         <x:v>AND gate</x:v>
       </x:c>
@@ -1376,14 +1293,14 @@
       <x:c r="B41" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C41" s="13" t="str">
+      <x:c r="C41" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bugs_addsubz","Add/sub")</x:f>
         <x:v>Add/sub</x:v>
       </x:c>
       <x:c r="D41" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E41" s="40" t="str">
+      <x:c r="E41" s="6" t="str">
         <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
         <x:v>Combined questions PDF</x:v>
       </x:c>
@@ -1395,7 +1312,7 @@
       <x:c r="B42" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C42" s="13" t="str">
+      <x:c r="C42" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4h","Wire")</x:f>
         <x:v>Wire</x:v>
       </x:c>
@@ -1413,14 +1330,14 @@
       <x:c r="B43" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C43" s="13" t="str">
+      <x:c r="C43" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4a","D Latch")</x:f>
         <x:v>D Latch</x:v>
       </x:c>
       <x:c r="D43" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E43" s="40" t="str">
+      <x:c r="E43" s="6" t="str">
         <x:f>HYPERLINK("HDLBits_Combined_Questions_and_Day2_Review.pdf","Combined questions PDF")</x:f>
         <x:v>Combined questions PDF</x:v>
       </x:c>
@@ -1432,7 +1349,7 @@
       <x:c r="B44" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C44" s="13" t="str">
+      <x:c r="C44" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm3onehot","Simple one-hot state transitions 3")</x:f>
         <x:v>Simple one-hot state transitions 3</x:v>
       </x:c>
@@ -1450,7 +1367,7 @@
       <x:c r="B45" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C45" s="13" t="str">
+      <x:c r="C45" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/norgate","NOR gate")</x:f>
         <x:v>NOR gate</x:v>
       </x:c>
@@ -1468,7 +1385,7 @@
       <x:c r="B46" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C46" s="13" t="str">
+      <x:c r="C46" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4i","GND")</x:f>
         <x:v>GND</x:v>
       </x:c>
@@ -1486,7 +1403,7 @@
       <x:c r="B47" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C47" s="13" t="str">
+      <x:c r="C47" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4b","DFF")</x:f>
         <x:v>DFF</x:v>
       </x:c>
@@ -1504,7 +1421,7 @@
       <x:c r="B48" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C48" s="13" t="str">
+      <x:c r="C48" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm3","Simple FSM 3 (asynchronous reset)")</x:f>
         <x:v>Simple FSM 3 (asynchronous reset)</x:v>
       </x:c>
@@ -1522,7 +1439,7 @@
       <x:c r="B49" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C49" s="13" t="str">
+      <x:c r="C49" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/xnorgate","XNOR gate")</x:f>
         <x:v>XNOR gate</x:v>
       </x:c>
@@ -1540,7 +1457,7 @@
       <x:c r="B50" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C50" s="13" t="str">
+      <x:c r="C50" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4e","NOR")</x:f>
         <x:v>NOR</x:v>
       </x:c>
@@ -1558,7 +1475,7 @@
       <x:c r="B51" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C51" s="13" t="str">
+      <x:c r="C51" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4c","DFF")</x:f>
         <x:v>DFF</x:v>
       </x:c>
@@ -1576,7 +1493,7 @@
       <x:c r="B52" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C52" s="13" t="str">
+      <x:c r="C52" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_case","Case statement")</x:f>
         <x:v>Case statement</x:v>
       </x:c>
@@ -1594,7 +1511,7 @@
       <x:c r="B53" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C53" s="13" t="str">
+      <x:c r="C53" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm3s","Simple FSM 3 (synchronous reset)")</x:f>
         <x:v>Simple FSM 3 (synchronous reset)</x:v>
       </x:c>
@@ -1612,7 +1529,7 @@
       <x:c r="B54" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C54" s="13" t="str">
+      <x:c r="C54" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/wire_decl","Declaring wires")</x:f>
         <x:v>Declaring wires</x:v>
       </x:c>
@@ -1630,7 +1547,7 @@
       <x:c r="B55" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C55" s="13" t="str">
+      <x:c r="C55" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4f","Another gate")</x:f>
         <x:v>Another gate</x:v>
       </x:c>
@@ -1648,15 +1565,15 @@
       <x:c r="B56" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C56" s="13" t="str">
+      <x:c r="C56" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4d","DFF+gate")</x:f>
         <x:v>DFF+gate</x:v>
       </x:c>
       <x:c r="D56" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E56" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="E56" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="22.049999237060547" customHeight="1">
@@ -1666,15 +1583,15 @@
       <x:c r="B57" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C57" s="13" t="str">
+      <x:c r="C57" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4g","Two gates")</x:f>
         <x:v>Two gates</x:v>
       </x:c>
       <x:c r="D57" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E57" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="E57" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="22.049999237060547" customHeight="1">
@@ -1684,15 +1601,15 @@
       <x:c r="B58" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C58" s="13" t="str">
+      <x:c r="C58" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/7458","7458 chip")</x:f>
         <x:v>7458 chip</x:v>
       </x:c>
       <x:c r="D58" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E58" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="E58" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="22.049999237060547" customHeight="1">
@@ -1702,14 +1619,14 @@
       <x:c r="B59" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C59" s="13" t="str">
+      <x:c r="C59" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q4","Design a Moore FSM")</x:f>
         <x:v>Design a Moore FSM</x:v>
       </x:c>
       <x:c r="D59" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E59" s="46" t="str">
+      <x:c r="E59" s="23" t="str">
         <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
@@ -1721,15 +1638,15 @@
       <x:c r="B60" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C60" s="13" t="str">
+      <x:c r="C60" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit1","Combinational circuit 1")</x:f>
         <x:v>Combinational circuit 1</x:v>
       </x:c>
       <x:c r="D60" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E60" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="E60" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="22.049999237060547" customHeight="1">
@@ -1739,15 +1656,15 @@
       <x:c r="B61" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C61" s="13" t="str">
+      <x:c r="C61" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mt2015_muxdff","Mux and DFF")</x:f>
         <x:v>Mux and DFF</x:v>
       </x:c>
-      <x:c r="D61" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E61" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D61" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E61" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="22.049999237060547" customHeight="1">
@@ -1757,15 +1674,15 @@
       <x:c r="B62" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C62" s="13" t="str">
+      <x:c r="C62" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gates","More logic gates")</x:f>
         <x:v>More logic gates</x:v>
       </x:c>
-      <x:c r="D62" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E62" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D62" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E62" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="22.049999237060547" customHeight="1">
@@ -1775,15 +1692,15 @@
       <x:c r="B63" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C63" s="13" t="str">
+      <x:c r="C63" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector0","Vectors")</x:f>
         <x:v>Vectors</x:v>
       </x:c>
-      <x:c r="D63" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E63" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D63" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E63" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="22.049999237060547" customHeight="1">
@@ -1793,15 +1710,15 @@
       <x:c r="B64" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C64" s="13" t="str">
+      <x:c r="C64" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_onehot","One-hot FSM")</x:f>
         <x:v>One-hot FSM</x:v>
       </x:c>
-      <x:c r="D64" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E64" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D64" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E64" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="22.049999237060547" customHeight="1">
@@ -1811,15 +1728,15 @@
       <x:c r="B65" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C65" s="13" t="str">
+      <x:c r="C65" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q4a","Mux and DFF")</x:f>
         <x:v>Mux and DFF</x:v>
       </x:c>
-      <x:c r="D65" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E65" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D65" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E65" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="22.049999237060547" customHeight="1">
@@ -1829,15 +1746,15 @@
       <x:c r="B66" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C66" s="13" t="str">
+      <x:c r="C66" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/7420","7420 chip")</x:f>
         <x:v>7420 chip</x:v>
       </x:c>
-      <x:c r="D66" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E66" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D66" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E66" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="22.049999237060547" customHeight="1">
@@ -1847,15 +1764,15 @@
       <x:c r="B67" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C67" s="13" t="str">
+      <x:c r="C67" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector1","Vectors in more detail")</x:f>
         <x:v>Vectors in more detail</x:v>
       </x:c>
-      <x:c r="D67" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E67" s="35" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D67" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E67" s="18" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="22.049999237060547" customHeight="1">
@@ -1865,15 +1782,15 @@
       <x:c r="B68" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C68" s="13" t="str">
+      <x:c r="C68" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit2","Combinational circuit 2")</x:f>
         <x:v>Combinational circuit 2</x:v>
       </x:c>
-      <x:c r="D68" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E68" s="23" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D68" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E68" s="15" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="22.049999237060547" customHeight="1">
@@ -1883,15 +1800,15 @@
       <x:c r="B69" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C69" s="13" t="str">
+      <x:c r="C69" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_ps2","PS/2 packet parser")</x:f>
         <x:v>PS/2 packet parser</x:v>
       </x:c>
-      <x:c r="D69" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E69" s="23" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D69" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E69" s="15" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="22.049999237060547" customHeight="1">
@@ -1901,15 +1818,15 @@
       <x:c r="B70" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C70" s="13" t="str">
+      <x:c r="C70" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/truthtable1","Truth tables")</x:f>
         <x:v>Truth tables</x:v>
       </x:c>
-      <x:c r="D70" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E70" s="23" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D70" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E70" s="15" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="22.049999237060547" customHeight="1">
@@ -1919,14 +1836,14 @@
       <x:c r="B71" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C71" s="13" t="str">
+      <x:c r="C71" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q4","DFFs and gates")</x:f>
         <x:v>DFFs and gates</x:v>
       </x:c>
-      <x:c r="D71" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E71" s="27" t="str">
+      <x:c r="D71" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E71" s="16" t="str">
         <x:f>HYPERLINK("HDLBits_Day4_Questions_Vector_DFF_PS2.pdf","Day 4 questions PDF")</x:f>
         <x:v>Day 4 questions PDF</x:v>
       </x:c>
@@ -1938,14 +1855,14 @@
       <x:c r="B72" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C72" s="13" t="str">
+      <x:c r="C72" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector2","Vector part select")</x:f>
         <x:v>Vector part select</x:v>
       </x:c>
-      <x:c r="D72" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E72" s="27" t="str">
+      <x:c r="D72" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E72" s="16" t="str">
         <x:f>HYPERLINK("HDLBits_Day4_Questions_Vector_DFF_PS2.pdf","Day 4 questions PDF")</x:f>
         <x:v>Day 4 questions PDF</x:v>
       </x:c>
@@ -1957,15 +1874,15 @@
       <x:c r="B73" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C73" s="13" t="str">
+      <x:c r="C73" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mt2015_eq2","Two-bit equality")</x:f>
         <x:v>Two-bit equality</x:v>
       </x:c>
-      <x:c r="D73" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E73" s="23" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D73" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E73" s="15" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="22.049999237060547" customHeight="1">
@@ -1975,15 +1892,15 @@
       <x:c r="B74" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C74" s="13" t="str">
+      <x:c r="C74" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q7","Create circuit from truth table")</x:f>
         <x:v>Create circuit from truth table</x:v>
       </x:c>
-      <x:c r="D74" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E74" s="23" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D74" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E74" s="15" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="22.049999237060547" customHeight="1">
@@ -1993,14 +1910,14 @@
       <x:c r="B75" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C75" s="13" t="str">
+      <x:c r="C75" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fsm_ps2data","PS/2 packet parser and datapath")</x:f>
         <x:v>PS/2 packet parser and datapath</x:v>
       </x:c>
-      <x:c r="D75" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E75" s="27" t="str">
+      <x:c r="D75" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E75" s="16" t="str">
         <x:f>HYPERLINK("HDLBits_Day4_Questions_Vector_DFF_PS2.pdf","Day 4 questions PDF")</x:f>
         <x:v>Day 4 questions PDF</x:v>
       </x:c>
@@ -2012,15 +1929,15 @@
       <x:c r="B76" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C76" s="13" t="str">
+      <x:c r="C76" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit3","Combinational circuit 3")</x:f>
         <x:v>Combinational circuit 3</x:v>
       </x:c>
-      <x:c r="D76" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E76" s="31" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D76" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E76" s="17" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="22.049999237060547" customHeight="1">
@@ -2030,15 +1947,15 @@
       <x:c r="B77" s="4" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C77" s="13" t="str">
+      <x:c r="C77" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mt2015_q4a","Simple circuit A")</x:f>
         <x:v>Simple circuit A</x:v>
       </x:c>
-      <x:c r="D77" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E77" s="31" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D77" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E77" s="17" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="22.049999237060547" customHeight="1">
@@ -2048,15 +1965,15 @@
       <x:c r="B78" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C78" s="13" t="str">
+      <x:c r="C78" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vectorgates","Bitwise operators")</x:f>
         <x:v>Bitwise operators</x:v>
       </x:c>
-      <x:c r="D78" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E78" s="31" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D78" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E78" s="17" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="22.049999237060547" customHeight="1">
@@ -2066,14 +1983,14 @@
       <x:c r="B79" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C79" s="13" t="str">
+      <x:c r="C79" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/edgedetect","Detect an edge")</x:f>
         <x:v>Detect an edge</x:v>
       </x:c>
-      <x:c r="D79" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E79" s="46" t="str">
+      <x:c r="D79" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E79" s="23" t="str">
         <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
@@ -2085,14 +2002,14 @@
       <x:c r="B80" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C80" s="13" t="str">
+      <x:c r="C80" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q8","Q8: Design a Mealy FSM")</x:f>
         <x:v>Q8: Design a Mealy FSM</x:v>
       </x:c>
-      <x:c r="D80" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E80" s="46" t="str">
+      <x:c r="D80" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E80" s="23" t="str">
         <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
@@ -2104,15 +2021,15 @@
       <x:c r="B81" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C81" s="13" t="str">
+      <x:c r="C81" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mt2015_q4b","Simple circuit B")</x:f>
         <x:v>Simple circuit B</x:v>
       </x:c>
-      <x:c r="D81" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E81" s="31" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D81" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E81" s="17" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="22.049999237060547" customHeight="1">
@@ -2122,14 +2039,14 @@
       <x:c r="B82" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C82" s="13" t="str">
+      <x:c r="C82" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gates4","Four-input gates")</x:f>
         <x:v>Four-input gates</x:v>
       </x:c>
-      <x:c r="D82" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E82" s="46" t="str">
+      <x:c r="D82" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E82" s="23" t="str">
         <x:f>HYPERLINK("HDLBits_Recovered_Code_Questions_54_74_75_77.pdf","Recovered questions PDF")</x:f>
         <x:v>Recovered questions PDF</x:v>
       </x:c>
@@ -2141,15 +2058,15 @@
       <x:c r="B83" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C83" s="13" t="str">
+      <x:c r="C83" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/edgedetect2","Detect both edges")</x:f>
         <x:v>Detect both edges</x:v>
       </x:c>
-      <x:c r="D83" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E83" s="31" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D83" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E83" s="17" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="22.049999237060547" customHeight="1">
@@ -2159,15 +2076,15 @@
       <x:c r="B84" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C84" s="13" t="str">
+      <x:c r="C84" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mt2015_q4","Combine circuits A and B")</x:f>
         <x:v>Combine circuits A and B</x:v>
       </x:c>
-      <x:c r="D84" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E84" s="31" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D84" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E84" s="17" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="22.049999237060547" customHeight="1">
@@ -2177,14 +2094,14 @@
       <x:c r="B85" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C85" s="13" t="str">
+      <x:c r="C85" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q5a","Q5a: Serial two's complementer (Moore FSM)")</x:f>
         <x:v>Q5a: Serial two's complementer (Moore FSM)</x:v>
       </x:c>
-      <x:c r="D85" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E85" s="42" t="str">
+      <x:c r="D85" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E85" s="22" t="str">
         <x:f>HYPERLINK("HDLBits_Entry80_Moore_Serial_Twos_Complement_Deep_Dive.pdf","Entry 80 Moore FSM PDF")</x:f>
         <x:v>Entry 80 Moore FSM PDF</x:v>
       </x:c>
@@ -2196,14 +2113,14 @@
       <x:c r="B86" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C86" s="13" t="str">
+      <x:c r="C86" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit4","Combinational circuit 4")</x:f>
         <x:v>Combinational circuit 4</x:v>
       </x:c>
-      <x:c r="D86" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E86" s="42" t="str">
+      <x:c r="D86" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E86" s="22" t="str">
         <x:f>HYPERLINK("HDLBits_Day5_Original_Submissions_Review.md","Day 5 submission review")</x:f>
         <x:v>Day 5 submission review</x:v>
       </x:c>
@@ -2215,14 +2132,14 @@
       <x:c r="B87" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C87" s="13" t="str">
+      <x:c r="C87" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector3","Vector concatenation operator")</x:f>
         <x:v>Vector concatenation operator</x:v>
       </x:c>
-      <x:c r="D87" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E87" s="42" t="str">
+      <x:c r="D87" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E87" s="22" t="str">
         <x:f>HYPERLINK("HDLBits_Day5_Original_Submissions_Review.md","Day 5 submission review")</x:f>
         <x:v>Day 5 submission review</x:v>
       </x:c>
@@ -2234,14 +2151,14 @@
       <x:c r="B88" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C88" s="13" t="str">
+      <x:c r="C88" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/edgecapture","Edge capture register")</x:f>
         <x:v>Edge capture register</x:v>
       </x:c>
-      <x:c r="D88" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E88" s="42" t="str">
+      <x:c r="D88" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E88" s="22" t="str">
         <x:f>HYPERLINK("HDLBits_Day5_Original_Submissions_Review.md","Day 5 submission review")</x:f>
         <x:v>Day 5 submission review</x:v>
       </x:c>
@@ -2253,14 +2170,14 @@
       <x:c r="B89" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C89" s="13" t="str">
+      <x:c r="C89" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/ringer","Ring or vibrate?")</x:f>
         <x:v>Ring or vibrate?</x:v>
       </x:c>
-      <x:c r="D89" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E89" s="42" t="str">
+      <x:c r="D89" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E89" s="22" t="str">
         <x:f>HYPERLINK("HDLBits_Day5_Original_Submissions_Review.md","Day 5 submission review")</x:f>
         <x:v>Day 5 submission review</x:v>
       </x:c>
@@ -2272,14 +2189,14 @@
       <x:c r="B90" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C90" s="13" t="str">
+      <x:c r="C90" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q5b","Q5b: Serial two's complementer (Mealy FSM)")</x:f>
         <x:v>Q5b: Serial two's complementer (Mealy FSM)</x:v>
       </x:c>
-      <x:c r="D90" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E90" s="42" t="str">
+      <x:c r="D90" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E90" s="22" t="str">
         <x:f>HYPERLINK("HDLBits_Day5_Original_Submissions_Review.md","Day 5 submission review")</x:f>
         <x:v>Day 5 submission review</x:v>
       </x:c>
@@ -2291,15 +2208,15 @@
       <x:c r="B91" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C91" s="13" t="str">
+      <x:c r="C91" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vectorr","Vector reversal 1")</x:f>
         <x:v>Vector reversal 1</x:v>
       </x:c>
-      <x:c r="D91" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E91" s="50" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D91" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E91" s="24" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="22.049999237060547" customHeight="1">
@@ -2309,14 +2226,14 @@
       <x:c r="B92" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C92" s="13" t="str">
+      <x:c r="C92" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/dualedge","Dual-edge triggered flip-flop")</x:f>
         <x:v>Dual-edge triggered flip-flop</x:v>
       </x:c>
-      <x:c r="D92" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E92" s="54" t="str">
+      <x:c r="D92" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E92" s="25" t="str">
         <x:f>HYPERLINK("HDLBits_Day6_Non_FSM_QA_Dualedge_and_Circuit5.pdf","Day 6 non-FSM Q&amp;A")</x:f>
         <x:v>Day 6 non-FSM Q&amp;A</x:v>
       </x:c>
@@ -2328,15 +2245,15 @@
       <x:c r="B93" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C93" s="13" t="str">
+      <x:c r="C93" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/thermostat","Thermostat")</x:f>
         <x:v>Thermostat</x:v>
       </x:c>
-      <x:c r="D93" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E93" s="50" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D93" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E93" s="24" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="22.049999237060547" customHeight="1">
@@ -2346,14 +2263,14 @@
       <x:c r="B94" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C94" s="13" t="str">
+      <x:c r="C94" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit5","Combinational circuit 5")</x:f>
         <x:v>Combinational circuit 5</x:v>
       </x:c>
-      <x:c r="D94" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E94" s="54" t="str">
+      <x:c r="D94" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E94" s="25" t="str">
         <x:f>HYPERLINK("HDLBits_Day6_Non_FSM_QA_Dualedge_and_Circuit5.pdf","Day 6 non-FSM Q&amp;A")</x:f>
         <x:v>Day 6 non-FSM Q&amp;A</x:v>
       </x:c>
@@ -2365,14 +2282,14 @@
       <x:c r="B95" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C95" s="13" t="str">
+      <x:c r="C95" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q3fsm","Q3a: FSM")</x:f>
         <x:v>Q3a: FSM</x:v>
       </x:c>
-      <x:c r="D95" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E95" s="54" t="str">
+      <x:c r="D95" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E95" s="25" t="str">
         <x:f>HYPERLINK("HDLBits_Entry90_Exams_2014_Q3FSM_Three_Sample_Window_Deep_Dive.pdf","Q3FSM deep-dive PDF")</x:f>
         <x:v>Q3FSM deep-dive PDF</x:v>
       </x:c>
@@ -2384,15 +2301,15 @@
       <x:c r="B96" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C96" s="13" t="str">
+      <x:c r="C96" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector4","Replication operator")</x:f>
         <x:v>Replication operator</x:v>
       </x:c>
-      <x:c r="D96" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E96" s="50" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D96" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E96" s="24" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="22.049999237060547" customHeight="1">
@@ -2402,15 +2319,15 @@
       <x:c r="B97" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C97" s="13" t="str">
+      <x:c r="C97" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count15","Four-bit binary counter")</x:f>
         <x:v>Four-bit binary counter</x:v>
       </x:c>
-      <x:c r="D97" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E97" s="50" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D97" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E97" s="24" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="22.049999237060547" customHeight="1">
@@ -2420,15 +2337,15 @@
       <x:c r="B98" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C98" s="13" t="str">
+      <x:c r="C98" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/popcount3","3-bit population count")</x:f>
         <x:v>3-bit population count</x:v>
       </x:c>
-      <x:c r="D98" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E98" s="50" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D98" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E98" s="24" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="22.049999237060547" customHeight="1">
@@ -2438,14 +2355,16 @@
       <x:c r="B99" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C99" s="13" t="str">
+      <x:c r="C99" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gatesv","Gates and vectors")</x:f>
         <x:v>Gates and vectors</x:v>
       </x:c>
       <x:c r="D99" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E99" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E99" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="22.049999237060547" customHeight="1">
       <x:c r="A100" s="4">
@@ -2454,14 +2373,16 @@
       <x:c r="B100" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C100" s="13" t="str">
+      <x:c r="C100" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count10","Decade counter")</x:f>
         <x:v>Decade counter</x:v>
       </x:c>
       <x:c r="D100" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E100" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E100" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="22.049999237060547" customHeight="1">
       <x:c r="A101" s="4">
@@ -2470,14 +2391,16 @@
       <x:c r="B101" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C101" s="13" t="str">
+      <x:c r="C101" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/vector5","More replication")</x:f>
         <x:v>More replication</x:v>
       </x:c>
       <x:c r="D101" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E101" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E101" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="22.049999237060547" customHeight="1">
       <x:c r="A102" s="4">
@@ -2486,14 +2409,16 @@
       <x:c r="B102" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C102" s="13" t="str">
+      <x:c r="C102" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q3bfsm","Q3b: FSM")</x:f>
         <x:v>Q3b: FSM</x:v>
       </x:c>
       <x:c r="D102" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E102" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E102" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" ht="22.049999237060547" customHeight="1">
       <x:c r="A103" s="4">
@@ -2502,14 +2427,16 @@
       <x:c r="B103" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C103" s="13" t="str">
+      <x:c r="C103" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit6","Combinational circuit 6")</x:f>
         <x:v>Combinational circuit 6</x:v>
       </x:c>
       <x:c r="D103" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E103" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E103" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="22.049999237060547" customHeight="1">
       <x:c r="A104" s="4">
@@ -2518,14 +2445,16 @@
       <x:c r="B104" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C104" s="13" t="str">
+      <x:c r="C104" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/gatesv100","Even longer vectors")</x:f>
         <x:v>Even longer vectors</x:v>
       </x:c>
       <x:c r="D104" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E104" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E104" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="22.049999237060547" customHeight="1">
       <x:c r="A105" s="4">
@@ -2534,14 +2463,16 @@
       <x:c r="B105" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C105" s="13" t="str">
+      <x:c r="C105" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count1to10","Decade counter again")</x:f>
         <x:v>Decade counter again</x:v>
       </x:c>
       <x:c r="D105" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E105" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E105" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="22.049999237060547" customHeight="1">
       <x:c r="A106" s="4">
@@ -2550,14 +2481,16 @@
       <x:c r="B106" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C106" s="13" t="str">
+      <x:c r="C106" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module","Modules")</x:f>
         <x:v>Modules</x:v>
       </x:c>
       <x:c r="D106" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E106" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E106" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" ht="22.049999237060547" customHeight="1">
       <x:c r="A107" s="4">
@@ -2566,14 +2499,17 @@
       <x:c r="B107" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C107" s="13" t="str">
+      <x:c r="C107" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q3c","Q3c: FSM logic")</x:f>
         <x:v>Q3c: FSM logic</x:v>
       </x:c>
       <x:c r="D107" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E107" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E107" s="26" t="str">
+        <x:f>HYPERLINK("HDLBits_Day7_QA_FSM_Warnings_and_Counter_Interface.pdf","Day 7 Q&amp;A")</x:f>
+        <x:v>Day 7 Q&amp;A</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="22.049999237060547" customHeight="1">
       <x:c r="A108" s="4">
@@ -2582,14 +2518,16 @@
       <x:c r="B108" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C108" s="13" t="str">
+      <x:c r="C108" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux2to1","2-to-1 multiplexer")</x:f>
         <x:v>2-to-1 multiplexer</x:v>
       </x:c>
       <x:c r="D108" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E108" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E108" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="22.049999237060547" customHeight="1">
       <x:c r="A109" s="4">
@@ -2598,14 +2536,16 @@
       <x:c r="B109" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C109" s="13" t="str">
+      <x:c r="C109" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/countslow","Slow decade counter")</x:f>
         <x:v>Slow decade counter</x:v>
       </x:c>
       <x:c r="D109" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E109" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E109" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="110" ht="22.049999237060547" customHeight="1">
       <x:c r="A110" s="4">
@@ -2614,14 +2554,16 @@
       <x:c r="B110" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C110" s="13" t="str">
+      <x:c r="C110" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_pos","Connecting ports by position")</x:f>
         <x:v>Connecting ports by position</x:v>
       </x:c>
       <x:c r="D110" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E110" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E110" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="22.049999237060547" customHeight="1">
       <x:c r="A111" s="4">
@@ -2630,14 +2572,16 @@
       <x:c r="B111" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C111" s="13" t="str">
+      <x:c r="C111" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit7","Sequential circuit 7")</x:f>
         <x:v>Sequential circuit 7</x:v>
       </x:c>
       <x:c r="D111" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E111" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E111" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="112" ht="22.049999237060547" customHeight="1">
       <x:c r="A112" s="4">
@@ -2646,204 +2590,230 @@
       <x:c r="B112" s="4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C112" s="13" t="str">
+      <x:c r="C112" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q6b","Q6b: FSM next-state logic")</x:f>
         <x:v>Q6b: FSM next-state logic</x:v>
       </x:c>
       <x:c r="D112" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E112" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E112" s="26" t="str">
+        <x:f>HYPERLINK("HDLBits_Day7_QA_FSM_Warnings_and_Counter_Interface.pdf","Day 7 Q&amp;A")</x:f>
+        <x:v>Day 7 Q&amp;A</x:v>
+      </x:c>
     </x:row>
     <x:row r="113" ht="22.049999237060547" customHeight="1">
       <x:c r="A113" s="4">
         <x:v>108</x:v>
       </x:c>
       <x:c r="B113" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C113" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C113" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux2to1v","2-to-1 bus multiplexer")</x:f>
         <x:v>2-to-1 bus multiplexer</x:v>
       </x:c>
       <x:c r="D113" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E113" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E113" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="22.049999237060547" customHeight="1">
       <x:c r="A114" s="4">
         <x:v>109</x:v>
       </x:c>
       <x:c r="B114" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C114" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C114" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q7a","Counter 1-12")</x:f>
         <x:v>Counter 1-12</x:v>
       </x:c>
       <x:c r="D114" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E114" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E114" s="26" t="str">
+        <x:f>HYPERLINK("HDLBits_Day7_QA_FSM_Warnings_and_Counter_Interface.pdf","Day 7 Q&amp;A")</x:f>
+        <x:v>Day 7 Q&amp;A</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="22.049999237060547" customHeight="1">
       <x:c r="A115" s="4">
         <x:v>110</x:v>
       </x:c>
       <x:c r="B115" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C115" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C115" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_name","Connecting ports by name")</x:f>
         <x:v>Connecting ports by name</x:v>
       </x:c>
       <x:c r="D115" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E115" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E115" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="22.049999237060547" customHeight="1">
       <x:c r="A116" s="4">
         <x:v>111</x:v>
       </x:c>
       <x:c r="B116" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C116" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C116" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux9to1v","9-to-1 multiplexer")</x:f>
         <x:v>9-to-1 multiplexer</x:v>
       </x:c>
       <x:c r="D116" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E116" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E116" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="22.049999237060547" customHeight="1">
       <x:c r="A117" s="4">
         <x:v>112</x:v>
       </x:c>
       <x:c r="B117" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C117" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C117" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q6c","Q6c: FSM one-hot next-state logic")</x:f>
         <x:v>Q6c: FSM one-hot next-state logic</x:v>
       </x:c>
       <x:c r="D117" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E117" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E117" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="22.049999237060547" customHeight="1">
       <x:c r="A118" s="4">
         <x:v>113</x:v>
       </x:c>
       <x:c r="B118" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C118" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C118" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q7b","Counter 1000")</x:f>
         <x:v>Counter 1000</x:v>
       </x:c>
-      <x:c r="D118" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E118" s="7"/>
+      <x:c r="D118" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E118" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="119" ht="22.049999237060547" customHeight="1">
       <x:c r="A119" s="4">
         <x:v>114</x:v>
       </x:c>
       <x:c r="B119" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C119" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C119" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit8","Sequential circuit 8")</x:f>
         <x:v>Sequential circuit 8</x:v>
       </x:c>
-      <x:c r="D119" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E119" s="7"/>
+      <x:c r="D119" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E119" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="120" ht="22.049999237060547" customHeight="1">
       <x:c r="A120" s="4">
         <x:v>115</x:v>
       </x:c>
       <x:c r="B120" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C120" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C120" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux256to1","256-to-1 multiplexer")</x:f>
         <x:v>256-to-1 multiplexer</x:v>
       </x:c>
-      <x:c r="D120" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E120" s="7"/>
+      <x:c r="D120" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E120" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="121" ht="22.049999237060547" customHeight="1">
       <x:c r="A121" s="4">
         <x:v>116</x:v>
       </x:c>
       <x:c r="B121" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C121" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C121" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_shift","Three modules")</x:f>
         <x:v>Three modules</x:v>
       </x:c>
-      <x:c r="D121" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E121" s="7"/>
+      <x:c r="D121" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E121" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="22.049999237060547" customHeight="1">
       <x:c r="A122" s="4">
         <x:v>117</x:v>
       </x:c>
       <x:c r="B122" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C122" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C122" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q6","Q6: FSM")</x:f>
         <x:v>Q6: FSM</x:v>
       </x:c>
-      <x:c r="D122" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E122" s="7"/>
+      <x:c r="D122" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E122" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="22.049999237060547" customHeight="1">
       <x:c r="A123" s="4">
         <x:v>118</x:v>
       </x:c>
       <x:c r="B123" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C123" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C123" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/countbcd","4-digit decimal counter")</x:f>
         <x:v>4-digit decimal counter</x:v>
       </x:c>
-      <x:c r="D123" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E123" s="7"/>
+      <x:c r="D123" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E123" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="124" ht="22.049999237060547" customHeight="1">
       <x:c r="A124" s="4">
         <x:v>119</x:v>
       </x:c>
       <x:c r="B124" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C124" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C124" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux256to1v","256-to-1 4-bit multiplexer")</x:f>
         <x:v>256-to-1 4-bit multiplexer</x:v>
       </x:c>
       <x:c r="D124" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E124" s="7"/>
     </x:row>
@@ -2852,46 +2822,50 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="B125" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C125" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C125" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_shift8","Modules and vectors")</x:f>
         <x:v>Modules and vectors</x:v>
       </x:c>
-      <x:c r="D125" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E125" s="7"/>
+      <x:c r="D125" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E125" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="22.049999237060547" customHeight="1">
       <x:c r="A126" s="4">
         <x:v>121</x:v>
       </x:c>
       <x:c r="B126" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C126" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C126" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit9","Sequential circuit 9")</x:f>
         <x:v>Sequential circuit 9</x:v>
       </x:c>
-      <x:c r="D126" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E126" s="7"/>
+      <x:c r="D126" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E126" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="22.049999237060547" customHeight="1">
       <x:c r="A127" s="4">
         <x:v>122</x:v>
       </x:c>
       <x:c r="B127" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C127" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C127" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/hadd","Half adder")</x:f>
         <x:v>Half adder</x:v>
       </x:c>
       <x:c r="D127" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E127" s="7"/>
     </x:row>
@@ -2900,14 +2874,14 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="B128" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C128" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C128" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count_clock","12-hour clock")</x:f>
         <x:v>12-hour clock</x:v>
       </x:c>
       <x:c r="D128" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E128" s="7"/>
     </x:row>
@@ -2916,14 +2890,14 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="B129" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C129" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C129" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2012_q2fsm","Q2a: FSM")</x:f>
         <x:v>Q2a: FSM</x:v>
       </x:c>
       <x:c r="D129" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E129" s="7"/>
     </x:row>
@@ -2932,14 +2906,14 @@
         <x:v>125</x:v>
       </x:c>
       <x:c r="B130" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C130" s="13" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C130" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_add","Adder 1")</x:f>
         <x:v>Adder 1</x:v>
       </x:c>
       <x:c r="D130" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E130" s="7"/>
     </x:row>
@@ -2950,12 +2924,12 @@
       <x:c r="B131" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C131" s="13" t="str">
+      <x:c r="C131" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fadd","Full adder")</x:f>
         <x:v>Full adder</x:v>
       </x:c>
       <x:c r="D131" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E131" s="7"/>
     </x:row>
@@ -2966,12 +2940,12 @@
       <x:c r="B132" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C132" s="13" t="str">
+      <x:c r="C132" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/shift4","4-bit shift register")</x:f>
         <x:v>4-bit shift register</x:v>
       </x:c>
       <x:c r="D132" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E132" s="7"/>
     </x:row>
@@ -2982,12 +2956,12 @@
       <x:c r="B133" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C133" s="13" t="str">
+      <x:c r="C133" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2012_q2b","Q2b: One-hot FSM equations")</x:f>
         <x:v>Q2b: One-hot FSM equations</x:v>
       </x:c>
       <x:c r="D133" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E133" s="7"/>
     </x:row>
@@ -2998,12 +2972,12 @@
       <x:c r="B134" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C134" s="13" t="str">
+      <x:c r="C134" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_fadd","Adder 2")</x:f>
         <x:v>Adder 2</x:v>
       </x:c>
       <x:c r="D134" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E134" s="7"/>
     </x:row>
@@ -3014,12 +2988,12 @@
       <x:c r="B135" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C135" s="13" t="str">
+      <x:c r="C135" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/adder3","3-bit binary adder")</x:f>
         <x:v>3-bit binary adder</x:v>
       </x:c>
       <x:c r="D135" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E135" s="7"/>
     </x:row>
@@ -3030,12 +3004,12 @@
       <x:c r="B136" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C136" s="13" t="str">
+      <x:c r="C136" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/rotate100","Left/right rotator")</x:f>
         <x:v>Left/right rotator</x:v>
       </x:c>
       <x:c r="D136" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E136" s="7"/>
     </x:row>
@@ -3046,12 +3020,12 @@
       <x:c r="B137" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C137" s="13" t="str">
+      <x:c r="C137" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit10","Sequential circuit 10")</x:f>
         <x:v>Sequential circuit 10</x:v>
       </x:c>
       <x:c r="D137" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E137" s="7"/>
     </x:row>
@@ -3062,12 +3036,12 @@
       <x:c r="B138" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C138" s="13" t="str">
+      <x:c r="C138" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2013_q2afsm","Q2a: FSM")</x:f>
         <x:v>Q2a: FSM</x:v>
       </x:c>
       <x:c r="D138" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E138" s="7"/>
     </x:row>
@@ -3078,12 +3052,12 @@
       <x:c r="B139" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C139" s="13" t="str">
+      <x:c r="C139" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_cseladd","Carry-select adder")</x:f>
         <x:v>Carry-select adder</x:v>
       </x:c>
       <x:c r="D139" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E139" s="7"/>
     </x:row>
@@ -3094,12 +3068,12 @@
       <x:c r="B140" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C140" s="13" t="str">
+      <x:c r="C140" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4j","Adder")</x:f>
         <x:v>Adder</x:v>
       </x:c>
       <x:c r="D140" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E140" s="7"/>
     </x:row>
@@ -3110,12 +3084,12 @@
       <x:c r="B141" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C141" s="13" t="str">
+      <x:c r="C141" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/shift18","Left/right arithmetic shift by 1 or 8")</x:f>
         <x:v>Left/right arithmetic shift by 1 or 8</x:v>
       </x:c>
       <x:c r="D141" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E141" s="7"/>
     </x:row>
@@ -3126,12 +3100,12 @@
       <x:c r="B142" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C142" s="13" t="str">
+      <x:c r="C142" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q1c","Signed addition overflow")</x:f>
         <x:v>Signed addition overflow</x:v>
       </x:c>
       <x:c r="D142" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E142" s="7"/>
     </x:row>
@@ -3142,12 +3116,12 @@
       <x:c r="B143" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C143" s="13" t="str">
+      <x:c r="C143" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_addsub","Adder-subtractor")</x:f>
         <x:v>Adder-subtractor</x:v>
       </x:c>
       <x:c r="D143" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E143" s="7"/>
     </x:row>
@@ -3158,12 +3132,12 @@
       <x:c r="B144" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C144" s="13" t="str">
+      <x:c r="C144" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2013_q2bfsm","Q2b: Another FSM")</x:f>
         <x:v>Q2b: Another FSM</x:v>
       </x:c>
       <x:c r="D144" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E144" s="7"/>
     </x:row>
@@ -3174,12 +3148,12 @@
       <x:c r="B145" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C145" s="13" t="str">
+      <x:c r="C145" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/clock","Clock")</x:f>
         <x:v>Clock</x:v>
       </x:c>
       <x:c r="D145" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E145" s="7"/>
     </x:row>
@@ -3190,12 +3164,12 @@
       <x:c r="B146" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C146" s="13" t="str">
+      <x:c r="C146" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lfsr5","5-bit LFSR")</x:f>
         <x:v>5-bit LFSR</x:v>
       </x:c>
       <x:c r="D146" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E146" s="7"/>
     </x:row>
@@ -3206,12 +3180,12 @@
       <x:c r="B147" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C147" s="13" t="str">
+      <x:c r="C147" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/adder100","100-bit binary adder")</x:f>
         <x:v>100-bit binary adder</x:v>
       </x:c>
       <x:c r="D147" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E147" s="7"/>
     </x:row>
@@ -3222,12 +3196,12 @@
       <x:c r="B148" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C148" s="13" t="str">
+      <x:c r="C148" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/alwaysblock1","Always blocks (combinational)")</x:f>
         <x:v>Always blocks (combinational)</x:v>
       </x:c>
       <x:c r="D148" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E148" s="7"/>
     </x:row>
@@ -3238,12 +3212,12 @@
       <x:c r="B149" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C149" s="13" t="str">
+      <x:c r="C149" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_count1k","Counter with period 1000")</x:f>
         <x:v>Counter with period 1000</x:v>
       </x:c>
       <x:c r="D149" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E149" s="7"/>
     </x:row>
@@ -3254,12 +3228,12 @@
       <x:c r="B150" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C150" s="13" t="str">
+      <x:c r="C150" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mt2015_lfsr","3-bit LFSR")</x:f>
         <x:v>3-bit LFSR</x:v>
       </x:c>
       <x:c r="D150" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E150" s="7"/>
     </x:row>
@@ -3270,12 +3244,12 @@
       <x:c r="B151" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C151" s="13" t="str">
+      <x:c r="C151" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bcdadd4","4-digit BCD adder")</x:f>
         <x:v>4-digit BCD adder</x:v>
       </x:c>
       <x:c r="D151" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E151" s="7"/>
     </x:row>
@@ -3286,12 +3260,12 @@
       <x:c r="B152" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C152" s="13" t="str">
+      <x:c r="C152" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/alwaysblock2","Always blocks (clocked)")</x:f>
         <x:v>Always blocks (clocked)</x:v>
       </x:c>
       <x:c r="D152" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E152" s="7"/>
     </x:row>
@@ -3302,12 +3276,12 @@
       <x:c r="B153" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C153" s="13" t="str">
+      <x:c r="C153" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/tb1","Testbench1")</x:f>
         <x:v>Testbench1</x:v>
       </x:c>
       <x:c r="D153" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E153" s="7"/>
     </x:row>
@@ -3318,12 +3292,12 @@
       <x:c r="B154" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C154" s="13" t="str">
+      <x:c r="C154" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_shiftcount","4-bit shift register and down counter")</x:f>
         <x:v>4-bit shift register and down counter</x:v>
       </x:c>
       <x:c r="D154" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E154" s="7"/>
     </x:row>
@@ -3334,12 +3308,12 @@
       <x:c r="B155" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C155" s="13" t="str">
+      <x:c r="C155" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap1","3-variable")</x:f>
         <x:v>3-variable</x:v>
       </x:c>
       <x:c r="D155" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E155" s="7"/>
     </x:row>
@@ -3350,12 +3324,12 @@
       <x:c r="B156" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C156" s="13" t="str">
+      <x:c r="C156" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lfsr32","32-bit LFSR")</x:f>
         <x:v>32-bit LFSR</x:v>
       </x:c>
       <x:c r="D156" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E156" s="7"/>
     </x:row>
@@ -3366,12 +3340,12 @@
       <x:c r="B157" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C157" s="13" t="str">
+      <x:c r="C157" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_if","If statement")</x:f>
         <x:v>If statement</x:v>
       </x:c>
       <x:c r="D157" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E157" s="7"/>
     </x:row>
@@ -3382,12 +3356,12 @@
       <x:c r="B158" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C158" s="13" t="str">
+      <x:c r="C158" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap2","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
       <x:c r="D158" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E158" s="7"/>
     </x:row>
@@ -3398,12 +3372,12 @@
       <x:c r="B159" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C159" s="13" t="str">
+      <x:c r="C159" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4k","Shift register")</x:f>
         <x:v>Shift register</x:v>
       </x:c>
       <x:c r="D159" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E159" s="7"/>
     </x:row>
@@ -3414,12 +3388,12 @@
       <x:c r="B160" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C160" s="13" t="str">
+      <x:c r="C160" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsmseq","FSM: Sequence 1101 recognizer")</x:f>
         <x:v>FSM: Sequence 1101 recognizer</x:v>
       </x:c>
       <x:c r="D160" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E160" s="7"/>
     </x:row>
@@ -3430,12 +3404,12 @@
       <x:c r="B161" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C161" s="13" t="str">
+      <x:c r="C161" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/and","AND gate")</x:f>
         <x:v>AND gate</x:v>
       </x:c>
       <x:c r="D161" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E161" s="7"/>
     </x:row>
@@ -3446,12 +3420,12 @@
       <x:c r="B162" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C162" s="13" t="str">
+      <x:c r="C162" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap3","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
       <x:c r="D162" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E162" s="7"/>
     </x:row>
@@ -3462,12 +3436,12 @@
       <x:c r="B163" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C163" s="13" t="str">
+      <x:c r="C163" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_if2","If statement latches")</x:f>
         <x:v>If statement latches</x:v>
       </x:c>
       <x:c r="D163" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E163" s="7"/>
     </x:row>
@@ -3478,12 +3452,12 @@
       <x:c r="B164" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C164" s="13" t="str">
+      <x:c r="C164" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q4b","Shift register")</x:f>
         <x:v>Shift register</x:v>
       </x:c>
       <x:c r="D164" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E164" s="7"/>
     </x:row>
@@ -3494,12 +3468,12 @@
       <x:c r="B165" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C165" s="13" t="str">
+      <x:c r="C165" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsmshift","FSM: Enable shift register")</x:f>
         <x:v>FSM: Enable shift register</x:v>
       </x:c>
       <x:c r="D165" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E165" s="7"/>
     </x:row>
@@ -3510,12 +3484,12 @@
       <x:c r="B166" s="4" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C166" s="13" t="str">
+      <x:c r="C166" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap4","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
       <x:c r="D166" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E166" s="7"/>
     </x:row>
@@ -3526,12 +3500,12 @@
       <x:c r="B167" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C167" s="13" t="str">
+      <x:c r="C167" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bugs_case","Case statement")</x:f>
         <x:v>Case statement</x:v>
       </x:c>
       <x:c r="D167" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E167" s="7"/>
     </x:row>
@@ -3542,12 +3516,12 @@
       <x:c r="B168" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C168" s="13" t="str">
+      <x:c r="C168" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q12","3-input LUT")</x:f>
         <x:v>3-input LUT</x:v>
       </x:c>
       <x:c r="D168" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E168" s="7"/>
     </x:row>
@@ -3558,12 +3532,12 @@
       <x:c r="B169" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C169" s="13" t="str">
+      <x:c r="C169" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q2","Minimum SOP and POS")</x:f>
         <x:v>Minimum SOP and POS</x:v>
       </x:c>
       <x:c r="D169" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E169" s="7"/>
     </x:row>
@@ -3574,12 +3548,12 @@
       <x:c r="B170" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C170" s="13" t="str">
+      <x:c r="C170" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsm","FSM: The complete FSM")</x:f>
         <x:v>FSM: The complete FSM</x:v>
       </x:c>
       <x:c r="D170" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E170" s="7"/>
     </x:row>
@@ -3590,12 +3564,12 @@
       <x:c r="B171" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C171" s="13" t="str">
+      <x:c r="C171" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/tb2","Testbench2")</x:f>
         <x:v>Testbench2</x:v>
       </x:c>
       <x:c r="D171" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E171" s="7"/>
     </x:row>
@@ -3606,12 +3580,12 @@
       <x:c r="B172" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C172" s="13" t="str">
+      <x:c r="C172" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_case2","Priority encoder")</x:f>
         <x:v>Priority encoder</x:v>
       </x:c>
       <x:c r="D172" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E172" s="7"/>
     </x:row>
@@ -3622,12 +3596,12 @@
       <x:c r="B173" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C173" s="13" t="str">
+      <x:c r="C173" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/rule90","Rule 90")</x:f>
         <x:v>Rule 90</x:v>
       </x:c>
       <x:c r="D173" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E173" s="7"/>
     </x:row>
@@ -3638,12 +3612,12 @@
       <x:c r="B174" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C174" s="13" t="str">
+      <x:c r="C174" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q3","Karnaugh map")</x:f>
         <x:v>Karnaugh map</x:v>
       </x:c>
       <x:c r="D174" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E174" s="7"/>
     </x:row>
@@ -3654,12 +3628,12 @@
       <x:c r="B175" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C175" s="13" t="str">
+      <x:c r="C175" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fancytimer","The complete timer")</x:f>
         <x:v>The complete timer</x:v>
       </x:c>
       <x:c r="D175" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E175" s="7"/>
     </x:row>
@@ -3670,12 +3644,12 @@
       <x:c r="B176" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C176" s="13" t="str">
+      <x:c r="C176" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_casez","Priority encoder with casez")</x:f>
         <x:v>Priority encoder with casez</x:v>
       </x:c>
       <x:c r="D176" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E176" s="7"/>
     </x:row>
@@ -3686,12 +3660,12 @@
       <x:c r="B177" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C177" s="13" t="str">
+      <x:c r="C177" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/rule110","Rule 110")</x:f>
         <x:v>Rule 110</x:v>
       </x:c>
       <x:c r="D177" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E177" s="7"/>
     </x:row>
@@ -3702,12 +3676,12 @@
       <x:c r="B178" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C178" s="13" t="str">
+      <x:c r="C178" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2012_q1g","Karnaugh map")</x:f>
         <x:v>Karnaugh map</x:v>
       </x:c>
       <x:c r="D178" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E178" s="7"/>
     </x:row>
@@ -3718,12 +3692,12 @@
       <x:c r="B179" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C179" s="13" t="str">
+      <x:c r="C179" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/tff","T flip-flop")</x:f>
         <x:v>T flip-flop</x:v>
       </x:c>
       <x:c r="D179" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E179" s="7"/>
     </x:row>
@@ -3734,12 +3708,12 @@
       <x:c r="B180" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C180" s="13" t="str">
+      <x:c r="C180" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsmonehot","FSM: One-hot logic equations")</x:f>
         <x:v>FSM: One-hot logic equations</x:v>
       </x:c>
       <x:c r="D180" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E180" s="7"/>
     </x:row>
@@ -3750,12 +3724,12 @@
       <x:c r="B181" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C181" s="13" t="str">
+      <x:c r="C181" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_nolatches","Avoiding latches")</x:f>
         <x:v>Avoiding latches</x:v>
       </x:c>
       <x:c r="D181" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E181" s="7"/>
     </x:row>
@@ -3766,12 +3740,12 @@
       <x:c r="B182" s="4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C182" s="13" t="str">
+      <x:c r="C182" s="12" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/conwaylife","Conway's Game of Life 16x16")</x:f>
         <x:v>Conway's Game of Life 16x16</x:v>
       </x:c>
       <x:c r="D182" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E182" s="7"/>
     </x:row>
@@ -3782,12 +3756,12 @@
       <x:c r="B183" s="5" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C183" s="14" t="str">
+      <x:c r="C183" s="13" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q3","K-map implemented with a multiplexer")</x:f>
         <x:v>K-map implemented with a multiplexer</x:v>
       </x:c>
       <x:c r="D183" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E183" s="8"/>
     </x:row>
@@ -3811,7 +3785,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f73f4956c7e4a50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R518ae5b2cbbb4ab4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile missing Attempt 2 completions before 12-hour clock
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R8847ae000aab4e4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R2ee624a2d9ae4ea2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -608,13 +608,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="1" t="n">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D3" s="1" t="n">
-        <x:v>58</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
         <x:v>4</x:v>
@@ -2704,11 +2704,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q7b","Counter 1000")</x:f>
         <x:v>Counter 1000</x:v>
       </x:c>
-      <x:c r="D118" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E118" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D118" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E118" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="22.049999237060547" customHeight="1">
@@ -2722,11 +2722,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit8","Sequential circuit 8")</x:f>
         <x:v>Sequential circuit 8</x:v>
       </x:c>
-      <x:c r="D119" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E119" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D119" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E119" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="22.049999237060547" customHeight="1">
@@ -2740,11 +2740,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux256to1","256-to-1 multiplexer")</x:f>
         <x:v>256-to-1 multiplexer</x:v>
       </x:c>
-      <x:c r="D120" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E120" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D120" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E120" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="22.049999237060547" customHeight="1">
@@ -2758,11 +2758,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_shift","Three modules")</x:f>
         <x:v>Three modules</x:v>
       </x:c>
-      <x:c r="D121" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E121" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D121" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E121" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="22.049999237060547" customHeight="1">
@@ -2776,11 +2776,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q6","Q6: FSM")</x:f>
         <x:v>Q6: FSM</x:v>
       </x:c>
-      <x:c r="D122" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E122" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D122" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E122" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="22.049999237060547" customHeight="1">
@@ -2794,11 +2794,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/countbcd","4-digit decimal counter")</x:f>
         <x:v>4-digit decimal counter</x:v>
       </x:c>
-      <x:c r="D123" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E123" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D123" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E123" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="22.049999237060547" customHeight="1">
@@ -2812,10 +2812,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/mux256to1v","256-to-1 4-bit multiplexer")</x:f>
         <x:v>256-to-1 4-bit multiplexer</x:v>
       </x:c>
-      <x:c r="D124" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E124" s="7"/>
+      <x:c r="D124" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E124" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="22.049999237060547" customHeight="1">
       <x:c r="A125" s="4">
@@ -2828,11 +2830,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_shift8","Modules and vectors")</x:f>
         <x:v>Modules and vectors</x:v>
       </x:c>
-      <x:c r="D125" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E125" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D125" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E125" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="22.049999237060547" customHeight="1">
@@ -2846,11 +2848,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit9","Sequential circuit 9")</x:f>
         <x:v>Sequential circuit 9</x:v>
       </x:c>
-      <x:c r="D126" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E126" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D126" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E126" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="22.049999237060547" customHeight="1">
@@ -2864,10 +2866,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/hadd","Half adder")</x:f>
         <x:v>Half adder</x:v>
       </x:c>
-      <x:c r="D127" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E127" s="7"/>
+      <x:c r="D127" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E127" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="22.049999237060547" customHeight="1">
       <x:c r="A128" s="4">
@@ -3785,7 +3789,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R518ae5b2cbbb4ab4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68bfba096a654136"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Review Attempt 2 study notes and record progress through 155 completions
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R9b7537e2c2ff4e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R7a3787a7d6a547fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -607,14 +607,14 @@
       <x:c r="A3" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="n">
-        <x:v>140</x:v>
+      <x:c s="1" r="B3" t="n">
+        <x:v>155</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D3" s="1" t="n">
-        <x:v>38</x:v>
+      <x:c s="1" r="D3" t="n">
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
         <x:v>4</x:v>
@@ -2884,8 +2884,8 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/count_clock","12-hour clock")</x:f>
         <x:v>12-hour clock</x:v>
       </x:c>
-      <x:c r="D128" s="4" t="str">
-        <x:v>Done</x:v>
+      <x:c r="D128" s="4" t="s">
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E128" s="26" t="str">
         <x:f>HYPERLINK("HDLBits_Day8_QA_Wire_Reg_and_Shift_Reset.pdf","Day 8 Q&amp;A")</x:f>
@@ -2903,15 +2903,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2012_q2fsm","Q2a: FSM")</x:f>
         <x:v>Q2a: FSM</x:v>
       </x:c>
-      <x:c r="D129" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E129" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No questions asked</x:t>
-        </x:is>
+      <x:c r="D129" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E129" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="22.049999237060547" customHeight="1">
@@ -2925,15 +2921,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_add","Adder 1")</x:f>
         <x:v>Adder 1</x:v>
       </x:c>
-      <x:c r="D130" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E130" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No questions asked</x:t>
-        </x:is>
+      <x:c r="D130" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E130" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="22.049999237060547" customHeight="1">
@@ -2947,15 +2939,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/fadd","Full adder")</x:f>
         <x:v>Full adder</x:v>
       </x:c>
-      <x:c r="D131" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E131" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No questions asked</x:t>
-        </x:is>
+      <x:c r="D131" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E131" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="22.049999237060547" customHeight="1">
@@ -2969,10 +2957,8 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/shift4","4-bit shift register")</x:f>
         <x:v>4-bit shift register</x:v>
       </x:c>
-      <x:c r="D132" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Done</x:t>
-        </x:is>
+      <x:c r="D132" s="4" t="s">
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E132" s="26" t="str">
         <x:f>HYPERLINK("HDLBits_Day8_QA_Wire_Reg_and_Shift_Reset.pdf","Day 8 Q&amp;A")</x:f>
@@ -2991,9 +2977,11 @@
         <x:v>Q2b: One-hot FSM equations</x:v>
       </x:c>
       <x:c r="D133" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E133" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E133" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="134" ht="22.049999237060547" customHeight="1">
       <x:c r="A134" s="4">
@@ -3006,10 +2994,8 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_fadd","Adder 2")</x:f>
         <x:v>Adder 2</x:v>
       </x:c>
-      <x:c r="D134" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Done</x:t>
-        </x:is>
+      <x:c r="D134" s="4" t="s">
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E134" s="26" t="str">
         <x:f>HYPERLINK("HDLBits_Day8_QA_Wire_Reg_and_Shift_Reset.pdf","Day 8 Q&amp;A")</x:f>
@@ -3027,15 +3013,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/adder3","3-bit binary adder")</x:f>
         <x:v>3-bit binary adder</x:v>
       </x:c>
-      <x:c r="D135" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E135" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No questions asked</x:t>
-        </x:is>
+      <x:c r="D135" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E135" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="22.049999237060547" customHeight="1">
@@ -3049,11 +3031,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/rotate100","Left/right rotator")</x:f>
         <x:v>Left/right rotator</x:v>
       </x:c>
-      <x:c r="D136" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E136" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D136" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E136" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="22.049999237060547" customHeight="1">
@@ -3068,9 +3050,11 @@
         <x:v>Sequential circuit 10</x:v>
       </x:c>
       <x:c r="D137" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E137" s="7"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E137" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="138" ht="22.049999237060547" customHeight="1">
       <x:c r="A138" s="4">
@@ -3083,10 +3067,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2013_q2afsm","Q2a: FSM")</x:f>
         <x:v>Q2a: FSM</x:v>
       </x:c>
-      <x:c r="D138" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E138" s="7"/>
+      <x:c r="D138" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E138" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="139" ht="22.049999237060547" customHeight="1">
       <x:c r="A139" s="4">
@@ -3099,11 +3085,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_cseladd","Carry-select adder")</x:f>
         <x:v>Carry-select adder</x:v>
       </x:c>
-      <x:c r="D139" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E139" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D139" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E139" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="22.049999237060547" customHeight="1">
@@ -3117,11 +3103,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4j","Adder")</x:f>
         <x:v>Adder</x:v>
       </x:c>
-      <x:c r="D140" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E140" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D140" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E140" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="22.049999237060547" customHeight="1">
@@ -3135,11 +3121,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/shift18","Left/right arithmetic shift by 1 or 8")</x:f>
         <x:v>Left/right arithmetic shift by 1 or 8</x:v>
       </x:c>
-      <x:c r="D141" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E141" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D141" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E141" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="22.049999237060547" customHeight="1">
@@ -3153,11 +3139,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q1c","Signed addition overflow")</x:f>
         <x:v>Signed addition overflow</x:v>
       </x:c>
-      <x:c r="D142" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E142" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D142" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E142" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="22.049999237060547" customHeight="1">
@@ -3171,11 +3157,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/module_addsub","Adder-subtractor")</x:f>
         <x:v>Adder-subtractor</x:v>
       </x:c>
-      <x:c r="D143" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E143" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D143" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E143" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="22.049999237060547" customHeight="1">
@@ -3189,11 +3175,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2013_q2bfsm","Q2b: Another FSM")</x:f>
         <x:v>Q2b: Another FSM</x:v>
       </x:c>
-      <x:c r="D144" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E144" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D144" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E144" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="22.049999237060547" customHeight="1">
@@ -3207,11 +3193,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/clock","Clock")</x:f>
         <x:v>Clock</x:v>
       </x:c>
-      <x:c r="D145" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E145" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D145" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E145" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="22.049999237060547" customHeight="1">
@@ -3241,11 +3227,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/adder100","100-bit binary adder")</x:f>
         <x:v>100-bit binary adder</x:v>
       </x:c>
-      <x:c r="D147" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E147" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D147" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E147" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="22.049999237060547" customHeight="1">
@@ -3259,11 +3245,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/alwaysblock1","Always blocks (combinational)")</x:f>
         <x:v>Always blocks (combinational)</x:v>
       </x:c>
-      <x:c r="D148" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E148" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D148" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E148" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="22.049999237060547" customHeight="1">
@@ -3277,11 +3263,11 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_count1k","Counter with period 1000")</x:f>
         <x:v>Counter with period 1000</x:v>
       </x:c>
-      <x:c r="D149" s="4" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="E149" s="7" t="str">
-        <x:v>No questions asked</x:v>
+      <x:c r="D149" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E149" s="7" t="s">
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="22.049999237060547" customHeight="1">
@@ -3311,10 +3297,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bcdadd4","4-digit BCD adder")</x:f>
         <x:v>4-digit BCD adder</x:v>
       </x:c>
-      <x:c r="D151" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E151" s="7"/>
+      <x:c r="D151" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E151" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="22.049999237060547" customHeight="1">
       <x:c r="A152" s="4">
@@ -3327,10 +3315,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/alwaysblock2","Always blocks (clocked)")</x:f>
         <x:v>Always blocks (clocked)</x:v>
       </x:c>
-      <x:c r="D152" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E152" s="7"/>
+      <x:c r="D152" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E152" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="22.049999237060547" customHeight="1">
       <x:c r="A153" s="4">
@@ -3343,10 +3333,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/tb1","Testbench1")</x:f>
         <x:v>Testbench1</x:v>
       </x:c>
-      <x:c r="D153" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E153" s="7"/>
+      <x:c r="D153" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E153" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="154" ht="22.049999237060547" customHeight="1">
       <x:c r="A154" s="4">
@@ -3359,10 +3351,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_shiftcount","4-bit shift register and down counter")</x:f>
         <x:v>4-bit shift register and down counter</x:v>
       </x:c>
-      <x:c r="D154" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E154" s="7"/>
+      <x:c r="D154" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E154" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="155" ht="22.049999237060547" customHeight="1">
       <x:c r="A155" s="4">
@@ -3375,10 +3369,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap1","3-variable")</x:f>
         <x:v>3-variable</x:v>
       </x:c>
-      <x:c r="D155" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E155" s="7"/>
+      <x:c r="D155" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E155" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="156" ht="22.049999237060547" customHeight="1">
       <x:c r="A156" s="4">
@@ -3407,10 +3403,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_if","If statement")</x:f>
         <x:v>If statement</x:v>
       </x:c>
-      <x:c r="D157" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E157" s="7"/>
+      <x:c r="D157" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E157" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="158" ht="22.049999237060547" customHeight="1">
       <x:c r="A158" s="4">
@@ -3423,10 +3421,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap2","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
-      <x:c r="D158" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E158" s="7"/>
+      <x:c r="D158" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E158" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="159" ht="22.049999237060547" customHeight="1">
       <x:c r="A159" s="4">
@@ -3439,10 +3439,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q4k","Shift register")</x:f>
         <x:v>Shift register</x:v>
       </x:c>
-      <x:c r="D159" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E159" s="7"/>
+      <x:c r="D159" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E159" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="160" ht="22.049999237060547" customHeight="1">
       <x:c r="A160" s="4">
@@ -3455,10 +3457,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsmseq","FSM: Sequence 1101 recognizer")</x:f>
         <x:v>FSM: Sequence 1101 recognizer</x:v>
       </x:c>
-      <x:c r="D160" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E160" s="7"/>
+      <x:c s="4" r="D160" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c s="26" r="E160" t="str">
+        <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","1101 FSM cleanup (pp. 4-5)")</x:f>
+        <x:v>1101 FSM cleanup (pp. 4-5)</x:v>
+      </x:c>
     </x:row>
     <x:row r="161" ht="22.049999237060547" customHeight="1">
       <x:c r="A161" s="4">
@@ -3471,10 +3476,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/and","AND gate")</x:f>
         <x:v>AND gate</x:v>
       </x:c>
-      <x:c r="D161" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E161" s="7"/>
+      <x:c s="4" r="D161" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c s="7" r="E161" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="22.049999237060547" customHeight="1">
       <x:c r="A162" s="4">
@@ -3487,10 +3494,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap3","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
-      <x:c r="D162" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E162" s="7"/>
+      <x:c s="4" r="D162" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c s="7" r="E162" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="163" ht="22.049999237060547" customHeight="1">
       <x:c r="A163" s="4">
@@ -3503,10 +3512,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_if2","If statement latches")</x:f>
         <x:v>If statement latches</x:v>
       </x:c>
-      <x:c r="D163" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E163" s="7"/>
+      <x:c s="4" r="D163" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c s="26" r="E163" t="str">
+        <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","If statements and latches (pp. 1-3)")</x:f>
+        <x:v>If statements and latches (pp. 1-3)</x:v>
+      </x:c>
     </x:row>
     <x:row r="164" ht="22.049999237060547" customHeight="1">
       <x:c r="A164" s="4">
@@ -3848,7 +3860,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60fcb7c5a7d846c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cff62c36c4b42ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Index and polish all HDLBits Attempt 2 study documents
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -3461,8 +3461,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c s="26" r="E160" t="str">
-        <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","1101 FSM cleanup (pp. 4-5)")</x:f>
-        <x:v>1101 FSM cleanup (pp. 4-5)</x:v>
+        <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","1101 FSM cleanup (pp. 5-6)")</x:f>
+        <x:v>1101 FSM cleanup (pp. 5-6)</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="22.049999237060547" customHeight="1">
@@ -3516,8 +3516,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c s="26" r="E163" t="str">
-        <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","If statements and latches (pp. 1-3)")</x:f>
-        <x:v>If statements and latches (pp. 1-3)</x:v>
+        <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","If statements and latches (pp. 2-4)")</x:f>
+        <x:v>If statements and latches (pp. 2-4)</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="22.049999237060547" customHeight="1">

</xml_diff>

<commit_message>
Consolidate Day 10 Rule 90 and Rule 110 notes
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R7a3787a7d6a547fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R62a7596326254704"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -607,14 +607,14 @@
       <x:c r="A3" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c s="1" r="B3" t="n">
-        <x:v>155</x:v>
+      <x:c r="B3" s="1" t="n">
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c s="1" r="D3" t="n">
-        <x:v>23</x:v>
+      <x:c r="D3" s="1" t="n">
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
         <x:v>4</x:v>
@@ -3457,10 +3457,10 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsmseq","FSM: Sequence 1101 recognizer")</x:f>
         <x:v>FSM: Sequence 1101 recognizer</x:v>
       </x:c>
-      <x:c s="4" r="D160" t="str">
+      <x:c r="D160" s="4" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c s="26" r="E160" t="str">
+      <x:c r="E160" s="26" t="str">
         <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","1101 FSM cleanup (pp. 5-6)")</x:f>
         <x:v>1101 FSM cleanup (pp. 5-6)</x:v>
       </x:c>
@@ -3476,10 +3476,10 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/and","AND gate")</x:f>
         <x:v>AND gate</x:v>
       </x:c>
-      <x:c s="4" r="D161" t="str">
+      <x:c r="D161" s="4" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c s="7" r="E161" t="str">
+      <x:c r="E161" s="7" t="str">
         <x:v>No questions asked</x:v>
       </x:c>
     </x:row>
@@ -3494,10 +3494,10 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap3","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
-      <x:c s="4" r="D162" t="str">
+      <x:c r="D162" s="4" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c s="7" r="E162" t="str">
+      <x:c r="E162" s="7" t="str">
         <x:v>No questions asked</x:v>
       </x:c>
     </x:row>
@@ -3512,10 +3512,10 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_if2","If statement latches")</x:f>
         <x:v>If statement latches</x:v>
       </x:c>
-      <x:c s="4" r="D163" t="str">
+      <x:c r="D163" s="4" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c s="26" r="E163" t="str">
+      <x:c r="E163" s="26" t="str">
         <x:f>HYPERLINK("HDLBits_Day9_QA_Latches_and_Sequence_FSM.pdf","If statements and latches (pp. 2-4)")</x:f>
         <x:v>If statements and latches (pp. 2-4)</x:v>
       </x:c>
@@ -3531,10 +3531,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2014_q4b","Shift register")</x:f>
         <x:v>Shift register</x:v>
       </x:c>
-      <x:c r="D164" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E164" s="7"/>
+      <x:c r="D164" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E164" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="165" ht="22.049999237060547" customHeight="1">
       <x:c r="A165" s="4">
@@ -3547,10 +3549,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/review2015_fsmshift","FSM: Enable shift register")</x:f>
         <x:v>FSM: Enable shift register</x:v>
       </x:c>
-      <x:c r="D165" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E165" s="7"/>
+      <x:c r="D165" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E165" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="166" ht="22.049999237060547" customHeight="1">
       <x:c r="A166" s="4">
@@ -3563,10 +3567,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/kmap4","4-variable")</x:f>
         <x:v>4-variable</x:v>
       </x:c>
-      <x:c r="D166" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E166" s="7"/>
+      <x:c r="D166" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E166" s="7" t="str">
+        <x:f>HYPERLINK("HDLBits_Day10_Kmaps_Boolean_Forms_and_Rules90_110.pdf","Kmap4: | versus + (pp. 2-3)")</x:f>
+        <x:v>Kmap4: | versus + (pp. 2-3)</x:v>
+      </x:c>
     </x:row>
     <x:row r="167" ht="22.049999237060547" customHeight="1">
       <x:c r="A167" s="4">
@@ -3579,10 +3586,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/bugs_case","Case statement")</x:f>
         <x:v>Case statement</x:v>
       </x:c>
-      <x:c r="D167" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E167" s="7"/>
+      <x:c r="D167" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E167" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="168" ht="22.049999237060547" customHeight="1">
       <x:c r="A168" s="4">
@@ -3595,10 +3604,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q12","3-input LUT")</x:f>
         <x:v>3-input LUT</x:v>
       </x:c>
-      <x:c r="D168" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E168" s="7"/>
+      <x:c r="D168" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E168" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="169" ht="22.049999237060547" customHeight="1">
       <x:c r="A169" s="4">
@@ -3611,10 +3622,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q2","Minimum SOP and POS")</x:f>
         <x:v>Minimum SOP and POS</x:v>
       </x:c>
-      <x:c r="D169" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E169" s="7"/>
+      <x:c r="D169" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E169" s="7" t="str">
+        <x:f>HYPERLINK("HDLBits_Day10_Kmaps_Boolean_Forms_and_Rules90_110.pdf","SOP, POS and De Morgan's law (pp. 4-5)")</x:f>
+        <x:v>SOP, POS and De Morgan's law (pp. 4-5)</x:v>
+      </x:c>
     </x:row>
     <x:row r="170" ht="22.049999237060547" customHeight="1">
       <x:c r="A170" s="4">
@@ -3659,10 +3673,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_case2","Priority encoder")</x:f>
         <x:v>Priority encoder</x:v>
       </x:c>
-      <x:c r="D172" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E172" s="7"/>
+      <x:c r="D172" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E172" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="173" ht="22.049999237060547" customHeight="1">
       <x:c r="A173" s="4">
@@ -3675,10 +3691,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/rule90","Rule 90")</x:f>
         <x:v>Rule 90</x:v>
       </x:c>
-      <x:c r="D173" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E173" s="7"/>
+      <x:c r="D173" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E173" s="7" t="str">
+        <x:f>HYPERLINK("HDLBits_Day10_Kmaps_Boolean_Forms_and_Rules90_110.pdf","Rule 90: why nextVal is used (pp. 6-7)")</x:f>
+        <x:v>Rule 90: why nextVal is used (pp. 6-7)</x:v>
+      </x:c>
     </x:row>
     <x:row r="174" ht="22.049999237060547" customHeight="1">
       <x:c r="A174" s="4">
@@ -3691,10 +3710,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/m2014_q3","Karnaugh map")</x:f>
         <x:v>Karnaugh map</x:v>
       </x:c>
-      <x:c r="D174" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E174" s="7"/>
+      <x:c r="D174" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E174" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="175" ht="22.049999237060547" customHeight="1">
       <x:c r="A175" s="4">
@@ -3723,10 +3744,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_casez","Priority encoder with casez")</x:f>
         <x:v>Priority encoder with casez</x:v>
       </x:c>
-      <x:c r="D176" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E176" s="7"/>
+      <x:c r="D176" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E176" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="177" ht="22.049999237060547" customHeight="1">
       <x:c r="A177" s="4">
@@ -3739,10 +3762,13 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/rule110","Rule 110")</x:f>
         <x:v>Rule 110</x:v>
       </x:c>
-      <x:c r="D177" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E177" s="7"/>
+      <x:c r="D177" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E177" s="7" t="str">
+        <x:f>HYPERLINK("HDLBits_Day10_Kmaps_Boolean_Forms_and_Rules90_110.pdf","Rule 110: expression and nextval (pp. 8-9)")</x:f>
+        <x:v>Rule 110: expression and nextval (pp. 8-9)</x:v>
+      </x:c>
     </x:row>
     <x:row r="178" ht="22.049999237060547" customHeight="1">
       <x:c r="A178" s="4">
@@ -3755,10 +3781,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2012_q1g","Karnaugh map")</x:f>
         <x:v>Karnaugh map</x:v>
       </x:c>
-      <x:c r="D178" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E178" s="7"/>
+      <x:c r="D178" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E178" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="179" ht="22.049999237060547" customHeight="1">
       <x:c r="A179" s="4">
@@ -3771,10 +3799,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/tb/tff","T flip-flop")</x:f>
         <x:v>T flip-flop</x:v>
       </x:c>
-      <x:c r="D179" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E179" s="7"/>
+      <x:c r="D179" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E179" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="180" ht="22.049999237060547" customHeight="1">
       <x:c r="A180" s="4">
@@ -3803,10 +3833,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_nolatches","Avoiding latches")</x:f>
         <x:v>Avoiding latches</x:v>
       </x:c>
-      <x:c r="D181" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E181" s="7"/>
+      <x:c r="D181" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E181" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
     <x:row r="182" ht="22.049999237060547" customHeight="1">
       <x:c r="A182" s="4">
@@ -3835,10 +3867,12 @@
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2014_q3","K-map implemented with a multiplexer")</x:f>
         <x:v>K-map implemented with a multiplexer</x:v>
       </x:c>
-      <x:c r="D183" s="5" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E183" s="8"/>
+      <x:c r="D183" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="E183" s="7" t="str">
+        <x:v>No questions asked</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3860,7 +3894,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cff62c36c4b42ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4403da945bf43a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate Attempt 2 into ten question-indexed daily PDFs
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
+++ b/HDLBits Attempt 2/HDLBits_Attempt_2_Tracker_Simple.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="E7" s="30" t="inlineStr">
         <is>
-          <t>Serial discussion PDF</t>
+          <t>Day 01 - answer pp. 3-11</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="E9" s="30" t="inlineStr">
         <is>
-          <t>Serial discussion PDF</t>
+          <t>Day 01 - answer pp. 3-11</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="E11" s="30" t="inlineStr">
         <is>
-          <t>Serial discussion PDF</t>
+          <t>Day 01 - answer pp. 11-12</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 8</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="E13" s="32" t="inlineStr">
         <is>
-          <t>HDLC discussion PDF</t>
+          <t>Day 01 - answer pp. 13-27</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       </c>
       <c r="E18" s="31" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 7</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="E24" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E25" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="E26" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="E27" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="E28" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 3-4</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="E29" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="E30" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E31" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 3, 6</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E32" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="E33" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 2, 9</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E34" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 7</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="E35" s="33" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 5</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="E36" s="29" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 10</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="E41" s="29" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 02 - answer pp. 11</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="E43" s="29" t="inlineStr">
         <is>
-          <t>Combined questions PDF</t>
+          <t>Day 03 - answer pp. 2</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="E59" s="34" t="inlineStr">
         <is>
-          <t>Recovered questions PDF</t>
+          <t>Day 03 - answer pp. 3</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="E71" s="34" t="inlineStr">
         <is>
-          <t>Day 4 questions PDF</t>
+          <t>Day 04 - answer pp. 3</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="E72" s="34" t="inlineStr">
         <is>
-          <t>Day 4 questions PDF</t>
+          <t>Day 04 - answer pp. 2-3</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="E75" s="34" t="inlineStr">
         <is>
-          <t>Day 4 questions PDF</t>
+          <t>Day 04 - answer pp. 4-6</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="E79" s="34" t="inlineStr">
         <is>
-          <t>Recovered questions PDF</t>
+          <t>Day 05 - answer pp. 3</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="E80" s="34" t="inlineStr">
         <is>
-          <t>Recovered questions PDF</t>
+          <t>Day 05 - answer pp. 4</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="E82" s="34" t="inlineStr">
         <is>
-          <t>Recovered questions PDF</t>
+          <t>Day 05 - answer pp. 5</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="E85" s="34" t="inlineStr">
         <is>
-          <t>Entry 80 Moore FSM PDF</t>
+          <t>Day 05 - answer pp. 7-13</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="E86" s="34" t="inlineStr">
         <is>
-          <t>Day 5 submission review</t>
+          <t>Day 05 - answer pp. 17</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="E87" s="34" t="inlineStr">
         <is>
-          <t>Day 5 submission review</t>
+          <t>Day 05 - answer pp. 17</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="E88" s="34" t="inlineStr">
         <is>
-          <t>Day 5 submission review</t>
+          <t>Day 05 - answer pp. 18</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="E89" s="34" t="inlineStr">
         <is>
-          <t>Day 5 submission review</t>
+          <t>Day 05 - answer pp. 18</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="E90" s="34" t="inlineStr">
         <is>
-          <t>Day 5 submission review</t>
+          <t>Day 05 - answer pp. 18-19</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E92" s="34" t="inlineStr">
         <is>
-          <t>Day 6 non-FSM Q&amp;A</t>
+          <t>Day 06 - answer pp. 4-15</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="E94" s="34" t="inlineStr">
         <is>
-          <t>Day 6 non-FSM Q&amp;A</t>
+          <t>Day 06 - answer pp. 16-18</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="E95" s="34" t="inlineStr">
         <is>
-          <t>Q3FSM deep-dive PDF</t>
+          <t>Day 06 - answer pp. 21-31</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="E107" s="34" t="inlineStr">
         <is>
-          <t>Day 7 Q&amp;A</t>
+          <t>Day 07 - answer pp. 2-3</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="E112" s="34" t="inlineStr">
         <is>
-          <t>Day 7 Q&amp;A</t>
+          <t>Day 07 - answer pp. 4</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="E114" s="34" t="inlineStr">
         <is>
-          <t>Day 7 Q&amp;A</t>
+          <t>Day 07 - answer pp. 5</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="E128" s="34" t="inlineStr">
         <is>
-          <t>Day 8 Q&amp;A</t>
+          <t>Day 08 - answer pp. 5-6</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="E132" s="34" t="inlineStr">
         <is>
-          <t>Day 8 Q&amp;A</t>
+          <t>Day 08 - answer pp. 4</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="E134" s="34" t="inlineStr">
         <is>
-          <t>Day 8 Q&amp;A</t>
+          <t>Day 08 - answer pp. 2-3</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="E146" s="41" t="inlineStr">
         <is>
-          <t>5-bit LFSR and taps (pp. 3-6)</t>
+          <t>Day 10 - answer pp. 27-30</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="E149" s="29" t="inlineStr">
         <is>
-          <t>Period-1000 counter (p. 3)</t>
+          <t>Day 10 - answer pp. 13</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="E150" s="41" t="inlineStr">
         <is>
-          <t>3-bit LFSR circuit (pp. 7-9)</t>
+          <t>Day 10 - answer pp. 31-33</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="E154" s="36" t="inlineStr">
         <is>
-          <t>Shift/down register and priority (pp. 4-5)</t>
+          <t>Day 10 - answer pp. 14-15</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E156" s="41" t="inlineStr">
         <is>
-          <t>32-bit LFSR timing (pp. 10-11)</t>
+          <t>Day 10 - answer pp. 34-35</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="E160" s="38" t="inlineStr">
         <is>
-          <t>1101 detection and next_state (p. 6)</t>
+          <t>Day 10 - answer pp. 16</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="E163" s="38" t="inlineStr">
         <is>
-          <t>If statements and latches (pp. 2-4)</t>
+          <t>Day 09 - answer pp. 2-4</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3828,7 @@
       </c>
       <c r="E165" s="36" t="inlineStr">
         <is>
-          <t>Four-cycle enable and multiple drivers (p. 7)</t>
+          <t>Day 10 - answer pp. 17</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="E166" s="29" t="inlineStr">
         <is>
-          <t>Kmap4: | versus + (pp. 2-3)</t>
+          <t>Day 10 - answer pp. 4-5</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="E169" s="36" t="inlineStr">
         <is>
-          <t>SOP, POS and De Morgan's law (pp. 4-5)</t>
+          <t>Day 10 - answer pp. 6-7</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="E170" s="36" t="inlineStr">
         <is>
-          <t>Complete timer-controller FSM (pp. 8-11)</t>
+          <t>Day 10 - answer pp. 18-21</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="E173" s="36" t="inlineStr">
         <is>
-          <t>Rule 90: why nextVal is used (pp. 6-7)</t>
+          <t>Day 10 - answer pp. 8-9</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="E175" s="36" t="inlineStr">
         <is>
-          <t>Complete timer and exact timing (pp. 12-15)</t>
+          <t>Day 10 - answer pp. 22-25</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="E177" s="36" t="inlineStr">
         <is>
-          <t>Rule 110: expression and nextval (pp. 8-9)</t>
+          <t>Day 10 - answer pp. 10-11</t>
         </is>
       </c>
     </row>
@@ -4165,7 +4165,7 @@
       </c>
       <c r="E182" s="41" t="inlineStr">
         <is>
-          <t>Conway grid and timing (pp. 2-7)</t>
+          <t>Day 10 - answer pp. 37-42</t>
         </is>
       </c>
     </row>

</xml_diff>